<commit_message>
Fix Phase 1C lineage cache: rebuild from Talend .item files instead of Python source
</commit_message>
<xml_diff>
--- a/output/migration_report.xlsx
+++ b/output/migration_report.xlsx
@@ -455,7 +455,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>2</t>
         </is>
       </c>
     </row>
@@ -467,7 +467,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>151</t>
+          <t>152</t>
         </is>
       </c>
     </row>
@@ -479,7 +479,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>4</t>
         </is>
       </c>
     </row>
@@ -506,10 +506,10 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H4"/>
+  <dimension ref="A1:H3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="25" customWidth="1" min="1" max="1"/>
+    <col width="29" customWidth="1" min="1" max="1"/>
     <col width="10" customWidth="1" min="2" max="2"/>
     <col width="12" customWidth="1" min="3" max="3"/>
     <col width="12" customWidth="1" min="4" max="4"/>
@@ -564,25 +564,25 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>SC_AS400_To_DropZone_MD</t>
+          <t>J_EyeMed_CMS_837_DBLoad_ODS</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>1.0</t>
+          <t>0.17</t>
         </is>
       </c>
       <c r="C2" t="n">
-        <v>48</v>
+        <v>76</v>
       </c>
       <c r="D2" t="inlineStr"/>
       <c r="E2" t="inlineStr">
         <is>
-          <t>AMBER</t>
+          <t>GREEN</t>
         </is>
       </c>
       <c r="F2" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G2" t="inlineStr">
         <is>
@@ -590,31 +590,31 @@
         </is>
       </c>
       <c r="H2" t="n">
-        <v>40</v>
+        <v>16</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>SC_AS400_To_DropZone_MD</t>
+          <t>J_EyeMed_CMS_837_DBLoad_ODS</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>3.0</t>
+          <t>0.18</t>
         </is>
       </c>
       <c r="C3" t="n">
-        <v>48</v>
+        <v>76</v>
       </c>
       <c r="D3" t="inlineStr"/>
       <c r="E3" t="inlineStr">
         <is>
-          <t>AMBER</t>
+          <t>GREEN</t>
         </is>
       </c>
       <c r="F3" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G3" t="inlineStr">
         <is>
@@ -622,39 +622,7 @@
         </is>
       </c>
       <c r="H3" t="n">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>SC_AS400_To_DropZone_MD</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>3.1</t>
-        </is>
-      </c>
-      <c r="C4" t="n">
-        <v>55</v>
-      </c>
-      <c r="D4" t="inlineStr"/>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>AMBER</t>
-        </is>
-      </c>
-      <c r="F4" t="n">
-        <v>3</v>
-      </c>
-      <c r="G4" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="H4" t="n">
-        <v>40</v>
+        <v>16</v>
       </c>
     </row>
   </sheetData>
@@ -668,12 +636,12 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E40"/>
+  <dimension ref="A1:E15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="25" customWidth="1" min="1" max="1"/>
+    <col width="29" customWidth="1" min="1" max="1"/>
     <col width="10" customWidth="1" min="2" max="2"/>
-    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="11" customWidth="1" min="3" max="3"/>
     <col width="10" customWidth="1" min="4" max="4"/>
     <col width="60" customWidth="1" min="5" max="5"/>
   </cols>
@@ -708,7 +676,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>SC_AS400_To_DropZone_MD</t>
+          <t>J_EyeMed_CMS_837_DBLoad_ODS</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -727,17 +695,17 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>SC_AS400_To_DropZone_MD</t>
+          <t>J_EyeMed_CMS_837_DBLoad_ODS</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>HIGH</t>
+          <t>LOW</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>tLibraryLoad</t>
+          <t>tMap</t>
         </is>
       </c>
       <c r="D3" t="inlineStr"/>
@@ -746,7 +714,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>SC_AS400_To_DropZone_MD</t>
+          <t>J_EyeMed_CMS_837_DBLoad_ODS</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -765,7 +733,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>SC_AS400_To_DropZone_MD</t>
+          <t>J_EyeMed_CMS_837_DBLoad_ODS</t>
         </is>
       </c>
       <c r="B5" t="inlineStr"/>
@@ -784,7 +752,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>SC_AS400_To_DropZone_MD</t>
+          <t>J_EyeMed_CMS_837_DBLoad_ODS</t>
         </is>
       </c>
       <c r="B6" t="inlineStr"/>
@@ -803,7 +771,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>SC_AS400_To_DropZone_MD</t>
+          <t>J_EyeMed_CMS_837_DBLoad_ODS</t>
         </is>
       </c>
       <c r="B7" t="inlineStr"/>
@@ -822,83 +790,83 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>SC_AS400_To_DropZone_MD</t>
+          <t>J_EyeMed_CMS_837_DBLoad_ODS</t>
         </is>
       </c>
       <c r="B8" t="inlineStr"/>
       <c r="C8" t="inlineStr">
         <is>
-          <t>tLibraryLoad</t>
+          <t>tJava</t>
         </is>
       </c>
       <c r="D8" t="inlineStr"/>
       <c r="E8" t="inlineStr">
         <is>
-          <t>{'risk': 'HIGH', 'issue': 'External Library Dependency', 'recommendation': 'Validate cloud runtime compatibility'}</t>
+          <t>{'risk': 'HIGH', 'issue': 'Custom Java Code', 'recommendation': 'Requires manual remediation'}</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>SC_AS400_To_DropZone_MD</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr"/>
+          <t>J_EyeMed_CMS_837_DBLoad_ODS</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
       <c r="C9" t="inlineStr">
         <is>
           <t>tJava</t>
         </is>
       </c>
       <c r="D9" t="inlineStr"/>
-      <c r="E9" t="inlineStr">
-        <is>
-          <t>{'risk': 'HIGH', 'issue': 'Custom Java Code', 'recommendation': 'Requires manual remediation'}</t>
-        </is>
-      </c>
+      <c r="E9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>SC_AS400_To_DropZone_MD</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr"/>
+          <t>J_EyeMed_CMS_837_DBLoad_ODS</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>LOW</t>
+        </is>
+      </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>tJava</t>
+          <t>tMap</t>
         </is>
       </c>
       <c r="D10" t="inlineStr"/>
-      <c r="E10" t="inlineStr">
-        <is>
-          <t>{'risk': 'HIGH', 'issue': 'Custom Java Code', 'recommendation': 'Requires manual remediation'}</t>
-        </is>
-      </c>
+      <c r="E10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>SC_AS400_To_DropZone_MD</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr"/>
+          <t>J_EyeMed_CMS_837_DBLoad_ODS</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>tLibraryLoad</t>
+          <t>tJavaRow</t>
         </is>
       </c>
       <c r="D11" t="inlineStr"/>
-      <c r="E11" t="inlineStr">
-        <is>
-          <t>{'risk': 'HIGH', 'issue': 'External Library Dependency', 'recommendation': 'Validate cloud runtime compatibility'}</t>
-        </is>
-      </c>
+      <c r="E11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>SC_AS400_To_DropZone_MD</t>
+          <t>J_EyeMed_CMS_837_DBLoad_ODS</t>
         </is>
       </c>
       <c r="B12" t="inlineStr"/>
@@ -917,7 +885,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>SC_AS400_To_DropZone_MD</t>
+          <t>J_EyeMed_CMS_837_DBLoad_ODS</t>
         </is>
       </c>
       <c r="B13" t="inlineStr"/>
@@ -936,7 +904,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>SC_AS400_To_DropZone_MD</t>
+          <t>J_EyeMed_CMS_837_DBLoad_ODS</t>
         </is>
       </c>
       <c r="B14" t="inlineStr"/>
@@ -955,492 +923,17 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>SC_AS400_To_DropZone_MD</t>
-        </is>
-      </c>
-      <c r="B15" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
+          <t>J_EyeMed_CMS_837_DBLoad_ODS</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr"/>
       <c r="C15" t="inlineStr">
         <is>
           <t>tJava</t>
         </is>
       </c>
       <c r="D15" t="inlineStr"/>
-      <c r="E15" t="inlineStr"/>
-    </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>SC_AS400_To_DropZone_MD</t>
-        </is>
-      </c>
-      <c r="B16" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
-      <c r="C16" t="inlineStr">
-        <is>
-          <t>tLibraryLoad</t>
-        </is>
-      </c>
-      <c r="D16" t="inlineStr"/>
-      <c r="E16" t="inlineStr"/>
-    </row>
-    <row r="17">
-      <c r="A17" t="inlineStr">
-        <is>
-          <t>SC_AS400_To_DropZone_MD</t>
-        </is>
-      </c>
-      <c r="B17" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
-      <c r="C17" t="inlineStr">
-        <is>
-          <t>tJavaRow</t>
-        </is>
-      </c>
-      <c r="D17" t="inlineStr"/>
-      <c r="E17" t="inlineStr"/>
-    </row>
-    <row r="18">
-      <c r="A18" t="inlineStr">
-        <is>
-          <t>SC_AS400_To_DropZone_MD</t>
-        </is>
-      </c>
-      <c r="B18" t="inlineStr"/>
-      <c r="C18" t="inlineStr">
-        <is>
-          <t>tJava</t>
-        </is>
-      </c>
-      <c r="D18" t="inlineStr"/>
-      <c r="E18" t="inlineStr">
-        <is>
-          <t>{'risk': 'HIGH', 'issue': 'Custom Java Code', 'recommendation': 'Requires manual remediation'}</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" t="inlineStr">
-        <is>
-          <t>SC_AS400_To_DropZone_MD</t>
-        </is>
-      </c>
-      <c r="B19" t="inlineStr"/>
-      <c r="C19" t="inlineStr">
-        <is>
-          <t>tJava</t>
-        </is>
-      </c>
-      <c r="D19" t="inlineStr"/>
-      <c r="E19" t="inlineStr">
-        <is>
-          <t>{'risk': 'HIGH', 'issue': 'Custom Java Code', 'recommendation': 'Requires manual remediation'}</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" t="inlineStr">
-        <is>
-          <t>SC_AS400_To_DropZone_MD</t>
-        </is>
-      </c>
-      <c r="B20" t="inlineStr"/>
-      <c r="C20" t="inlineStr">
-        <is>
-          <t>tJava</t>
-        </is>
-      </c>
-      <c r="D20" t="inlineStr"/>
-      <c r="E20" t="inlineStr">
-        <is>
-          <t>{'risk': 'HIGH', 'issue': 'Custom Java Code', 'recommendation': 'Requires manual remediation'}</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" t="inlineStr">
-        <is>
-          <t>SC_AS400_To_DropZone_MD</t>
-        </is>
-      </c>
-      <c r="B21" t="inlineStr"/>
-      <c r="C21" t="inlineStr">
-        <is>
-          <t>tLibraryLoad</t>
-        </is>
-      </c>
-      <c r="D21" t="inlineStr"/>
-      <c r="E21" t="inlineStr">
-        <is>
-          <t>{'risk': 'HIGH', 'issue': 'External Library Dependency', 'recommendation': 'Validate cloud runtime compatibility'}</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" t="inlineStr">
-        <is>
-          <t>SC_AS400_To_DropZone_MD</t>
-        </is>
-      </c>
-      <c r="B22" t="inlineStr"/>
-      <c r="C22" t="inlineStr">
-        <is>
-          <t>tJava</t>
-        </is>
-      </c>
-      <c r="D22" t="inlineStr"/>
-      <c r="E22" t="inlineStr">
-        <is>
-          <t>{'risk': 'HIGH', 'issue': 'Custom Java Code', 'recommendation': 'Requires manual remediation'}</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" t="inlineStr">
-        <is>
-          <t>SC_AS400_To_DropZone_MD</t>
-        </is>
-      </c>
-      <c r="B23" t="inlineStr"/>
-      <c r="C23" t="inlineStr">
-        <is>
-          <t>tJava</t>
-        </is>
-      </c>
-      <c r="D23" t="inlineStr"/>
-      <c r="E23" t="inlineStr">
-        <is>
-          <t>{'risk': 'HIGH', 'issue': 'Custom Java Code', 'recommendation': 'Requires manual remediation'}</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" t="inlineStr">
-        <is>
-          <t>SC_AS400_To_DropZone_MD</t>
-        </is>
-      </c>
-      <c r="B24" t="inlineStr"/>
-      <c r="C24" t="inlineStr">
-        <is>
-          <t>tLibraryLoad</t>
-        </is>
-      </c>
-      <c r="D24" t="inlineStr"/>
-      <c r="E24" t="inlineStr">
-        <is>
-          <t>{'risk': 'HIGH', 'issue': 'External Library Dependency', 'recommendation': 'Validate cloud runtime compatibility'}</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" t="inlineStr">
-        <is>
-          <t>SC_AS400_To_DropZone_MD</t>
-        </is>
-      </c>
-      <c r="B25" t="inlineStr"/>
-      <c r="C25" t="inlineStr">
-        <is>
-          <t>tJava</t>
-        </is>
-      </c>
-      <c r="D25" t="inlineStr"/>
-      <c r="E25" t="inlineStr">
-        <is>
-          <t>{'risk': 'HIGH', 'issue': 'Custom Java Code', 'recommendation': 'Requires manual remediation'}</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" t="inlineStr">
-        <is>
-          <t>SC_AS400_To_DropZone_MD</t>
-        </is>
-      </c>
-      <c r="B26" t="inlineStr"/>
-      <c r="C26" t="inlineStr">
-        <is>
-          <t>tJava</t>
-        </is>
-      </c>
-      <c r="D26" t="inlineStr"/>
-      <c r="E26" t="inlineStr">
-        <is>
-          <t>{'risk': 'HIGH', 'issue': 'Custom Java Code', 'recommendation': 'Requires manual remediation'}</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" t="inlineStr">
-        <is>
-          <t>SC_AS400_To_DropZone_MD</t>
-        </is>
-      </c>
-      <c r="B27" t="inlineStr"/>
-      <c r="C27" t="inlineStr">
-        <is>
-          <t>tJava</t>
-        </is>
-      </c>
-      <c r="D27" t="inlineStr"/>
-      <c r="E27" t="inlineStr">
-        <is>
-          <t>{'risk': 'HIGH', 'issue': 'Custom Java Code', 'recommendation': 'Requires manual remediation'}</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" t="inlineStr">
-        <is>
-          <t>SC_AS400_To_DropZone_MD</t>
-        </is>
-      </c>
-      <c r="B28" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
-      <c r="C28" t="inlineStr">
-        <is>
-          <t>tJava</t>
-        </is>
-      </c>
-      <c r="D28" t="inlineStr"/>
-      <c r="E28" t="inlineStr"/>
-    </row>
-    <row r="29">
-      <c r="A29" t="inlineStr">
-        <is>
-          <t>SC_AS400_To_DropZone_MD</t>
-        </is>
-      </c>
-      <c r="B29" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
-      <c r="C29" t="inlineStr">
-        <is>
-          <t>tLibraryLoad</t>
-        </is>
-      </c>
-      <c r="D29" t="inlineStr"/>
-      <c r="E29" t="inlineStr"/>
-    </row>
-    <row r="30">
-      <c r="A30" t="inlineStr">
-        <is>
-          <t>SC_AS400_To_DropZone_MD</t>
-        </is>
-      </c>
-      <c r="B30" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
-      <c r="C30" t="inlineStr">
-        <is>
-          <t>tJavaRow</t>
-        </is>
-      </c>
-      <c r="D30" t="inlineStr"/>
-      <c r="E30" t="inlineStr"/>
-    </row>
-    <row r="31">
-      <c r="A31" t="inlineStr">
-        <is>
-          <t>SC_AS400_To_DropZone_MD</t>
-        </is>
-      </c>
-      <c r="B31" t="inlineStr"/>
-      <c r="C31" t="inlineStr">
-        <is>
-          <t>tJava</t>
-        </is>
-      </c>
-      <c r="D31" t="inlineStr"/>
-      <c r="E31" t="inlineStr">
-        <is>
-          <t>{'risk': 'HIGH', 'issue': 'Custom Java Code', 'recommendation': 'Requires manual remediation'}</t>
-        </is>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" t="inlineStr">
-        <is>
-          <t>SC_AS400_To_DropZone_MD</t>
-        </is>
-      </c>
-      <c r="B32" t="inlineStr"/>
-      <c r="C32" t="inlineStr">
-        <is>
-          <t>tJava</t>
-        </is>
-      </c>
-      <c r="D32" t="inlineStr"/>
-      <c r="E32" t="inlineStr">
-        <is>
-          <t>{'risk': 'HIGH', 'issue': 'Custom Java Code', 'recommendation': 'Requires manual remediation'}</t>
-        </is>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" t="inlineStr">
-        <is>
-          <t>SC_AS400_To_DropZone_MD</t>
-        </is>
-      </c>
-      <c r="B33" t="inlineStr"/>
-      <c r="C33" t="inlineStr">
-        <is>
-          <t>tJava</t>
-        </is>
-      </c>
-      <c r="D33" t="inlineStr"/>
-      <c r="E33" t="inlineStr">
-        <is>
-          <t>{'risk': 'HIGH', 'issue': 'Custom Java Code', 'recommendation': 'Requires manual remediation'}</t>
-        </is>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" t="inlineStr">
-        <is>
-          <t>SC_AS400_To_DropZone_MD</t>
-        </is>
-      </c>
-      <c r="B34" t="inlineStr"/>
-      <c r="C34" t="inlineStr">
-        <is>
-          <t>tLibraryLoad</t>
-        </is>
-      </c>
-      <c r="D34" t="inlineStr"/>
-      <c r="E34" t="inlineStr">
-        <is>
-          <t>{'risk': 'HIGH', 'issue': 'External Library Dependency', 'recommendation': 'Validate cloud runtime compatibility'}</t>
-        </is>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" t="inlineStr">
-        <is>
-          <t>SC_AS400_To_DropZone_MD</t>
-        </is>
-      </c>
-      <c r="B35" t="inlineStr"/>
-      <c r="C35" t="inlineStr">
-        <is>
-          <t>tJava</t>
-        </is>
-      </c>
-      <c r="D35" t="inlineStr"/>
-      <c r="E35" t="inlineStr">
-        <is>
-          <t>{'risk': 'HIGH', 'issue': 'Custom Java Code', 'recommendation': 'Requires manual remediation'}</t>
-        </is>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" t="inlineStr">
-        <is>
-          <t>SC_AS400_To_DropZone_MD</t>
-        </is>
-      </c>
-      <c r="B36" t="inlineStr"/>
-      <c r="C36" t="inlineStr">
-        <is>
-          <t>tJava</t>
-        </is>
-      </c>
-      <c r="D36" t="inlineStr"/>
-      <c r="E36" t="inlineStr">
-        <is>
-          <t>{'risk': 'HIGH', 'issue': 'Custom Java Code', 'recommendation': 'Requires manual remediation'}</t>
-        </is>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" t="inlineStr">
-        <is>
-          <t>SC_AS400_To_DropZone_MD</t>
-        </is>
-      </c>
-      <c r="B37" t="inlineStr"/>
-      <c r="C37" t="inlineStr">
-        <is>
-          <t>tLibraryLoad</t>
-        </is>
-      </c>
-      <c r="D37" t="inlineStr"/>
-      <c r="E37" t="inlineStr">
-        <is>
-          <t>{'risk': 'HIGH', 'issue': 'External Library Dependency', 'recommendation': 'Validate cloud runtime compatibility'}</t>
-        </is>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" t="inlineStr">
-        <is>
-          <t>SC_AS400_To_DropZone_MD</t>
-        </is>
-      </c>
-      <c r="B38" t="inlineStr"/>
-      <c r="C38" t="inlineStr">
-        <is>
-          <t>tJava</t>
-        </is>
-      </c>
-      <c r="D38" t="inlineStr"/>
-      <c r="E38" t="inlineStr">
-        <is>
-          <t>{'risk': 'HIGH', 'issue': 'Custom Java Code', 'recommendation': 'Requires manual remediation'}</t>
-        </is>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" t="inlineStr">
-        <is>
-          <t>SC_AS400_To_DropZone_MD</t>
-        </is>
-      </c>
-      <c r="B39" t="inlineStr"/>
-      <c r="C39" t="inlineStr">
-        <is>
-          <t>tJava</t>
-        </is>
-      </c>
-      <c r="D39" t="inlineStr"/>
-      <c r="E39" t="inlineStr">
-        <is>
-          <t>{'risk': 'HIGH', 'issue': 'Custom Java Code', 'recommendation': 'Requires manual remediation'}</t>
-        </is>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" t="inlineStr">
-        <is>
-          <t>SC_AS400_To_DropZone_MD</t>
-        </is>
-      </c>
-      <c r="B40" t="inlineStr"/>
-      <c r="C40" t="inlineStr">
-        <is>
-          <t>tJava</t>
-        </is>
-      </c>
-      <c r="D40" t="inlineStr"/>
-      <c r="E40" t="inlineStr">
+      <c r="E15" t="inlineStr">
         <is>
           <t>{'risk': 'HIGH', 'issue': 'Custom Java Code', 'recommendation': 'Requires manual remediation'}</t>
         </is>
@@ -1457,12 +950,12 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D152"/>
+  <dimension ref="A1:D153"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="25" customWidth="1" min="1" max="1"/>
+    <col width="29" customWidth="1" min="1" max="1"/>
     <col width="16" customWidth="1" min="2" max="2"/>
-    <col width="25" customWidth="1" min="3" max="3"/>
+    <col width="21" customWidth="1" min="3" max="3"/>
     <col width="10" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
@@ -1491,13 +984,13 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>SC_AS400_To_DropZone_MD</t>
+          <t>J_EyeMed_CMS_837_DBLoad_ODS</t>
         </is>
       </c>
       <c r="B2" t="inlineStr"/>
       <c r="C2" t="inlineStr">
         <is>
-          <t>tMysqlInput</t>
+          <t>tMSSqlConnection</t>
         </is>
       </c>
       <c r="D2" t="inlineStr"/>
@@ -1505,13 +998,13 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>SC_AS400_To_DropZone_MD</t>
+          <t>J_EyeMed_CMS_837_DBLoad_ODS</t>
         </is>
       </c>
       <c r="B3" t="inlineStr"/>
       <c r="C3" t="inlineStr">
         <is>
-          <t>tFlowToIterate</t>
+          <t>tFileList</t>
         </is>
       </c>
       <c r="D3" t="inlineStr"/>
@@ -1519,13 +1012,13 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>SC_AS400_To_DropZone_MD</t>
+          <t>J_EyeMed_CMS_837_DBLoad_ODS</t>
         </is>
       </c>
       <c r="B4" t="inlineStr"/>
       <c r="C4" t="inlineStr">
         <is>
-          <t>tJava</t>
+          <t>tFileInputRaw</t>
         </is>
       </c>
       <c r="D4" t="inlineStr"/>
@@ -1533,13 +1026,13 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>SC_AS400_To_DropZone_MD</t>
+          <t>J_EyeMed_CMS_837_DBLoad_ODS</t>
         </is>
       </c>
       <c r="B5" t="inlineStr"/>
       <c r="C5" t="inlineStr">
         <is>
-          <t>tJava</t>
+          <t>tHMap</t>
         </is>
       </c>
       <c r="D5" t="inlineStr"/>
@@ -1547,13 +1040,13 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>SC_AS400_To_DropZone_MD</t>
+          <t>J_EyeMed_CMS_837_DBLoad_ODS</t>
         </is>
       </c>
       <c r="B6" t="inlineStr"/>
       <c r="C6" t="inlineStr">
         <is>
-          <t>tFTPPut</t>
+          <t>tFileOutputRaw</t>
         </is>
       </c>
       <c r="D6" t="inlineStr"/>
@@ -1561,13 +1054,13 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>SC_AS400_To_DropZone_MD</t>
+          <t>J_EyeMed_CMS_837_DBLoad_ODS</t>
         </is>
       </c>
       <c r="B7" t="inlineStr"/>
       <c r="C7" t="inlineStr">
         <is>
-          <t>tAS400Input</t>
+          <t>tDie</t>
         </is>
       </c>
       <c r="D7" t="inlineStr"/>
@@ -1575,13 +1068,13 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>SC_AS400_To_DropZone_MD</t>
+          <t>J_EyeMed_CMS_837_DBLoad_ODS</t>
         </is>
       </c>
       <c r="B8" t="inlineStr"/>
       <c r="C8" t="inlineStr">
         <is>
-          <t>tFileOutputDelimited</t>
+          <t>tFileList</t>
         </is>
       </c>
       <c r="D8" t="inlineStr"/>
@@ -1589,13 +1082,13 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>SC_AS400_To_DropZone_MD</t>
+          <t>J_EyeMed_CMS_837_DBLoad_ODS</t>
         </is>
       </c>
       <c r="B9" t="inlineStr"/>
       <c r="C9" t="inlineStr">
         <is>
-          <t>tFTPConnection</t>
+          <t>tJava</t>
         </is>
       </c>
       <c r="D9" t="inlineStr"/>
@@ -1603,13 +1096,13 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>SC_AS400_To_DropZone_MD</t>
+          <t>J_EyeMed_CMS_837_DBLoad_ODS</t>
         </is>
       </c>
       <c r="B10" t="inlineStr"/>
       <c r="C10" t="inlineStr">
         <is>
-          <t>tPrejob</t>
+          <t>tMSSqlInput</t>
         </is>
       </c>
       <c r="D10" t="inlineStr"/>
@@ -1617,13 +1110,13 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>SC_AS400_To_DropZone_MD</t>
+          <t>J_EyeMed_CMS_837_DBLoad_ODS</t>
         </is>
       </c>
       <c r="B11" t="inlineStr"/>
       <c r="C11" t="inlineStr">
         <is>
-          <t>tJava</t>
+          <t>tMap</t>
         </is>
       </c>
       <c r="D11" t="inlineStr"/>
@@ -1631,13 +1124,13 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>SC_AS400_To_DropZone_MD</t>
+          <t>J_EyeMed_CMS_837_DBLoad_ODS</t>
         </is>
       </c>
       <c r="B12" t="inlineStr"/>
       <c r="C12" t="inlineStr">
         <is>
-          <t>tLibraryLoad</t>
+          <t>tSetGlobalVar</t>
         </is>
       </c>
       <c r="D12" t="inlineStr"/>
@@ -1645,13 +1138,13 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>SC_AS400_To_DropZone_MD</t>
+          <t>J_EyeMed_CMS_837_DBLoad_ODS</t>
         </is>
       </c>
       <c r="B13" t="inlineStr"/>
       <c r="C13" t="inlineStr">
         <is>
-          <t>tJava</t>
+          <t>tFileInputXML</t>
         </is>
       </c>
       <c r="D13" t="inlineStr"/>
@@ -1659,13 +1152,13 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>SC_AS400_To_DropZone_MD</t>
+          <t>J_EyeMed_CMS_837_DBLoad_ODS</t>
         </is>
       </c>
       <c r="B14" t="inlineStr"/>
       <c r="C14" t="inlineStr">
         <is>
-          <t>tFileDelete</t>
+          <t>tMap</t>
         </is>
       </c>
       <c r="D14" t="inlineStr"/>
@@ -1673,13 +1166,13 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>SC_AS400_To_DropZone_MD</t>
+          <t>J_EyeMed_CMS_837_DBLoad_ODS</t>
         </is>
       </c>
       <c r="B15" t="inlineStr"/>
       <c r="C15" t="inlineStr">
         <is>
-          <t>tJava</t>
+          <t>tMap</t>
         </is>
       </c>
       <c r="D15" t="inlineStr"/>
@@ -1687,13 +1180,13 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>SC_AS400_To_DropZone_MD</t>
+          <t>J_EyeMed_CMS_837_DBLoad_ODS</t>
         </is>
       </c>
       <c r="B16" t="inlineStr"/>
       <c r="C16" t="inlineStr">
         <is>
-          <t>tAS400Connection</t>
+          <t>tHashInput</t>
         </is>
       </c>
       <c r="D16" t="inlineStr"/>
@@ -1701,13 +1194,13 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>SC_AS400_To_DropZone_MD</t>
+          <t>J_EyeMed_CMS_837_DBLoad_ODS</t>
         </is>
       </c>
       <c r="B17" t="inlineStr"/>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Implicit_context_joblet</t>
+          <t>tMSSqlOutput</t>
         </is>
       </c>
       <c r="D17" t="inlineStr"/>
@@ -1715,13 +1208,13 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>SC_AS400_To_DropZone_MD</t>
+          <t>J_EyeMed_CMS_837_DBLoad_ODS</t>
         </is>
       </c>
       <c r="B18" t="inlineStr"/>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Job_Start</t>
+          <t>tFileInputXML</t>
         </is>
       </c>
       <c r="D18" t="inlineStr"/>
@@ -1729,13 +1222,13 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>SC_AS400_To_DropZone_MD</t>
+          <t>J_EyeMed_CMS_837_DBLoad_ODS</t>
         </is>
       </c>
       <c r="B19" t="inlineStr"/>
       <c r="C19" t="inlineStr">
         <is>
-          <t>tMysqlConnection</t>
+          <t>tMap</t>
         </is>
       </c>
       <c r="D19" t="inlineStr"/>
@@ -1743,13 +1236,13 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>SC_AS400_To_DropZone_MD</t>
+          <t>J_EyeMed_CMS_837_DBLoad_ODS</t>
         </is>
       </c>
       <c r="B20" t="inlineStr"/>
       <c r="C20" t="inlineStr">
         <is>
-          <t>tFixedFlowInput</t>
+          <t>tMap</t>
         </is>
       </c>
       <c r="D20" t="inlineStr"/>
@@ -1757,13 +1250,13 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>SC_AS400_To_DropZone_MD</t>
+          <t>J_EyeMed_CMS_837_DBLoad_ODS</t>
         </is>
       </c>
       <c r="B21" t="inlineStr"/>
       <c r="C21" t="inlineStr">
         <is>
-          <t>tLogRow</t>
+          <t>tHashInput</t>
         </is>
       </c>
       <c r="D21" t="inlineStr"/>
@@ -1771,13 +1264,13 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>SC_AS400_To_DropZone_MD</t>
+          <t>J_EyeMed_CMS_837_DBLoad_ODS</t>
         </is>
       </c>
       <c r="B22" t="inlineStr"/>
       <c r="C22" t="inlineStr">
         <is>
-          <t>tMysqlOutput</t>
+          <t>tMSSqlOutput</t>
         </is>
       </c>
       <c r="D22" t="inlineStr"/>
@@ -1785,13 +1278,13 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>SC_AS400_To_DropZone_MD</t>
+          <t>J_EyeMed_CMS_837_DBLoad_ODS</t>
         </is>
       </c>
       <c r="B23" t="inlineStr"/>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Job_End</t>
+          <t>tFileInputXML</t>
         </is>
       </c>
       <c r="D23" t="inlineStr"/>
@@ -1799,13 +1292,13 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>SC_AS400_To_DropZone_MD</t>
+          <t>J_EyeMed_CMS_837_DBLoad_ODS</t>
         </is>
       </c>
       <c r="B24" t="inlineStr"/>
       <c r="C24" t="inlineStr">
         <is>
-          <t>tMysqlInput</t>
+          <t>tMap</t>
         </is>
       </c>
       <c r="D24" t="inlineStr"/>
@@ -1813,13 +1306,13 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>SC_AS400_To_DropZone_MD</t>
+          <t>J_EyeMed_CMS_837_DBLoad_ODS</t>
         </is>
       </c>
       <c r="B25" t="inlineStr"/>
       <c r="C25" t="inlineStr">
         <is>
-          <t>tJavaRow</t>
+          <t>tMap</t>
         </is>
       </c>
       <c r="D25" t="inlineStr"/>
@@ -1827,13 +1320,13 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>SC_AS400_To_DropZone_MD</t>
+          <t>J_EyeMed_CMS_837_DBLoad_ODS</t>
         </is>
       </c>
       <c r="B26" t="inlineStr"/>
       <c r="C26" t="inlineStr">
         <is>
-          <t>tDie</t>
+          <t>tHashInput</t>
         </is>
       </c>
       <c r="D26" t="inlineStr"/>
@@ -1841,13 +1334,13 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>SC_AS400_To_DropZone_MD</t>
+          <t>J_EyeMed_CMS_837_DBLoad_ODS</t>
         </is>
       </c>
       <c r="B27" t="inlineStr"/>
       <c r="C27" t="inlineStr">
         <is>
-          <t>tDie</t>
+          <t>tMSSqlOutput</t>
         </is>
       </c>
       <c r="D27" t="inlineStr"/>
@@ -1855,13 +1348,13 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>SC_AS400_To_DropZone_MD</t>
+          <t>J_EyeMed_CMS_837_DBLoad_ODS</t>
         </is>
       </c>
       <c r="B28" t="inlineStr"/>
       <c r="C28" t="inlineStr">
         <is>
-          <t>tDie</t>
+          <t>tFixedFlowInput</t>
         </is>
       </c>
       <c r="D28" t="inlineStr"/>
@@ -1869,13 +1362,13 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>SC_AS400_To_DropZone_MD</t>
+          <t>J_EyeMed_CMS_837_DBLoad_ODS</t>
         </is>
       </c>
       <c r="B29" t="inlineStr"/>
       <c r="C29" t="inlineStr">
         <is>
-          <t>tLibraryLoad</t>
+          <t>tJavaRow</t>
         </is>
       </c>
       <c r="D29" t="inlineStr"/>
@@ -1883,13 +1376,13 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>SC_AS400_To_DropZone_MD</t>
+          <t>J_EyeMed_CMS_837_DBLoad_ODS</t>
         </is>
       </c>
       <c r="B30" t="inlineStr"/>
       <c r="C30" t="inlineStr">
         <is>
-          <t>tMysqlInput</t>
+          <t>tFileList</t>
         </is>
       </c>
       <c r="D30" t="inlineStr"/>
@@ -1897,13 +1390,13 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>SC_AS400_To_DropZone_MD</t>
+          <t>J_EyeMed_CMS_837_DBLoad_ODS</t>
         </is>
       </c>
       <c r="B31" t="inlineStr"/>
       <c r="C31" t="inlineStr">
         <is>
-          <t>tFlowToIterate</t>
+          <t>tFileCopy</t>
         </is>
       </c>
       <c r="D31" t="inlineStr"/>
@@ -1911,13 +1404,13 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>SC_AS400_To_DropZone_MD</t>
+          <t>J_EyeMed_CMS_837_DBLoad_ODS</t>
         </is>
       </c>
       <c r="B32" t="inlineStr"/>
       <c r="C32" t="inlineStr">
         <is>
-          <t>tMysqlInput</t>
+          <t>tJava</t>
         </is>
       </c>
       <c r="D32" t="inlineStr"/>
@@ -1925,13 +1418,13 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>SC_AS400_To_DropZone_MD</t>
+          <t>J_EyeMed_CMS_837_DBLoad_ODS</t>
         </is>
       </c>
       <c r="B33" t="inlineStr"/>
       <c r="C33" t="inlineStr">
         <is>
-          <t>tJavaRow</t>
+          <t>tSendMail</t>
         </is>
       </c>
       <c r="D33" t="inlineStr"/>
@@ -1939,13 +1432,13 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>SC_AS400_To_DropZone_MD</t>
+          <t>J_EyeMed_CMS_837_DBLoad_ODS</t>
         </is>
       </c>
       <c r="B34" t="inlineStr"/>
       <c r="C34" t="inlineStr">
         <is>
-          <t>tDie</t>
+          <t>tFileInputXML</t>
         </is>
       </c>
       <c r="D34" t="inlineStr"/>
@@ -1953,13 +1446,13 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>SC_AS400_To_DropZone_MD</t>
+          <t>J_EyeMed_CMS_837_DBLoad_ODS</t>
         </is>
       </c>
       <c r="B35" t="inlineStr"/>
       <c r="C35" t="inlineStr">
         <is>
-          <t>tJava</t>
+          <t>tMap</t>
         </is>
       </c>
       <c r="D35" t="inlineStr"/>
@@ -1967,13 +1460,13 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>SC_AS400_To_DropZone_MD</t>
+          <t>J_EyeMed_CMS_837_DBLoad_ODS</t>
         </is>
       </c>
       <c r="B36" t="inlineStr"/>
       <c r="C36" t="inlineStr">
         <is>
-          <t>tPostjob</t>
+          <t>tMap</t>
         </is>
       </c>
       <c r="D36" t="inlineStr"/>
@@ -1981,13 +1474,13 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>SC_AS400_To_DropZone_MD</t>
+          <t>J_EyeMed_CMS_837_DBLoad_ODS</t>
         </is>
       </c>
       <c r="B37" t="inlineStr"/>
       <c r="C37" t="inlineStr">
         <is>
-          <t>tAS400Close</t>
+          <t>tMSSqlOutput</t>
         </is>
       </c>
       <c r="D37" t="inlineStr"/>
@@ -1995,13 +1488,13 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>SC_AS400_To_DropZone_MD</t>
+          <t>J_EyeMed_CMS_837_DBLoad_ODS</t>
         </is>
       </c>
       <c r="B38" t="inlineStr"/>
       <c r="C38" t="inlineStr">
         <is>
-          <t>tMysqlClose</t>
+          <t>tFileInputDelimited</t>
         </is>
       </c>
       <c r="D38" t="inlineStr"/>
@@ -2009,13 +1502,13 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>SC_AS400_To_DropZone_MD</t>
+          <t>J_EyeMed_CMS_837_DBLoad_ODS</t>
         </is>
       </c>
       <c r="B39" t="inlineStr"/>
       <c r="C39" t="inlineStr">
         <is>
-          <t>tJava</t>
+          <t>tJavaRow</t>
         </is>
       </c>
       <c r="D39" t="inlineStr"/>
@@ -2023,13 +1516,13 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>SC_AS400_To_DropZone_MD</t>
+          <t>J_EyeMed_CMS_837_DBLoad_ODS</t>
         </is>
       </c>
       <c r="B40" t="inlineStr"/>
       <c r="C40" t="inlineStr">
         <is>
-          <t>tMysqlInput</t>
+          <t>tFileInputXML</t>
         </is>
       </c>
       <c r="D40" t="inlineStr"/>
@@ -2037,13 +1530,13 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>SC_AS400_To_DropZone_MD</t>
+          <t>J_EyeMed_CMS_837_DBLoad_ODS</t>
         </is>
       </c>
       <c r="B41" t="inlineStr"/>
       <c r="C41" t="inlineStr">
         <is>
-          <t>tJavaRow</t>
+          <t>tMap</t>
         </is>
       </c>
       <c r="D41" t="inlineStr"/>
@@ -2051,13 +1544,13 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>SC_AS400_To_DropZone_MD</t>
+          <t>J_EyeMed_CMS_837_DBLoad_ODS</t>
         </is>
       </c>
       <c r="B42" t="inlineStr"/>
       <c r="C42" t="inlineStr">
         <is>
-          <t>tJava</t>
+          <t>tMap</t>
         </is>
       </c>
       <c r="D42" t="inlineStr"/>
@@ -2065,13 +1558,13 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>SC_AS400_To_DropZone_MD</t>
+          <t>J_EyeMed_CMS_837_DBLoad_ODS</t>
         </is>
       </c>
       <c r="B43" t="inlineStr"/>
       <c r="C43" t="inlineStr">
         <is>
-          <t>tFileDelete</t>
+          <t>tMSSqlInput</t>
         </is>
       </c>
       <c r="D43" t="inlineStr"/>
@@ -2079,13 +1572,13 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>SC_AS400_To_DropZone_MD</t>
+          <t>J_EyeMed_CMS_837_DBLoad_ODS</t>
         </is>
       </c>
       <c r="B44" t="inlineStr"/>
       <c r="C44" t="inlineStr">
         <is>
-          <t>tFixedFlowInput</t>
+          <t>tMSSqlOutput</t>
         </is>
       </c>
       <c r="D44" t="inlineStr"/>
@@ -2093,13 +1586,13 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>SC_AS400_To_DropZone_MD</t>
+          <t>J_EyeMed_CMS_837_DBLoad_ODS</t>
         </is>
       </c>
       <c r="B45" t="inlineStr"/>
       <c r="C45" t="inlineStr">
         <is>
-          <t>tLogRow</t>
+          <t>tFTPConnection</t>
         </is>
       </c>
       <c r="D45" t="inlineStr"/>
@@ -2107,13 +1600,13 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>SC_AS400_To_DropZone_MD</t>
+          <t>J_EyeMed_CMS_837_DBLoad_ODS</t>
         </is>
       </c>
       <c r="B46" t="inlineStr"/>
       <c r="C46" t="inlineStr">
         <is>
-          <t>tMysqlOutput</t>
+          <t>tFTPFileList</t>
         </is>
       </c>
       <c r="D46" t="inlineStr"/>
@@ -2121,13 +1614,13 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>SC_AS400_To_DropZone_MD</t>
+          <t>J_EyeMed_CMS_837_DBLoad_ODS</t>
         </is>
       </c>
       <c r="B47" t="inlineStr"/>
       <c r="C47" t="inlineStr">
         <is>
-          <t>Job_End</t>
+          <t>tFTPGet</t>
         </is>
       </c>
       <c r="D47" t="inlineStr"/>
@@ -2135,13 +1628,13 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>SC_AS400_To_DropZone_MD</t>
+          <t>J_EyeMed_CMS_837_DBLoad_ODS</t>
         </is>
       </c>
       <c r="B48" t="inlineStr"/>
       <c r="C48" t="inlineStr">
         <is>
-          <t>tFTPClose</t>
+          <t>tSendMail</t>
         </is>
       </c>
       <c r="D48" t="inlineStr"/>
@@ -2149,13 +1642,13 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>SC_AS400_To_DropZone_MD</t>
+          <t>J_EyeMed_CMS_837_DBLoad_ODS</t>
         </is>
       </c>
       <c r="B49" t="inlineStr"/>
       <c r="C49" t="inlineStr">
         <is>
-          <t>Job_Error</t>
+          <t>tSendMail</t>
         </is>
       </c>
       <c r="D49" t="inlineStr"/>
@@ -2163,13 +1656,13 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>SC_AS400_To_DropZone_MD</t>
+          <t>J_EyeMed_CMS_837_DBLoad_ODS</t>
         </is>
       </c>
       <c r="B50" t="inlineStr"/>
       <c r="C50" t="inlineStr">
         <is>
-          <t>tMysqlInput</t>
+          <t>tDie</t>
         </is>
       </c>
       <c r="D50" t="inlineStr"/>
@@ -2177,13 +1670,13 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>SC_AS400_To_DropZone_MD</t>
+          <t>J_EyeMed_CMS_837_DBLoad_ODS</t>
         </is>
       </c>
       <c r="B51" t="inlineStr"/>
       <c r="C51" t="inlineStr">
         <is>
-          <t>tFlowToIterate</t>
+          <t>tPrejob</t>
         </is>
       </c>
       <c r="D51" t="inlineStr"/>
@@ -2191,13 +1684,13 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>SC_AS400_To_DropZone_MD</t>
+          <t>J_EyeMed_CMS_837_DBLoad_ODS</t>
         </is>
       </c>
       <c r="B52" t="inlineStr"/>
       <c r="C52" t="inlineStr">
         <is>
-          <t>tJava</t>
+          <t>tMSSqlConnection</t>
         </is>
       </c>
       <c r="D52" t="inlineStr"/>
@@ -2205,13 +1698,13 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>SC_AS400_To_DropZone_MD</t>
+          <t>J_EyeMed_CMS_837_DBLoad_ODS</t>
         </is>
       </c>
       <c r="B53" t="inlineStr"/>
       <c r="C53" t="inlineStr">
         <is>
-          <t>tJava</t>
+          <t>tStatCatcher</t>
         </is>
       </c>
       <c r="D53" t="inlineStr"/>
@@ -2219,13 +1712,13 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>SC_AS400_To_DropZone_MD</t>
+          <t>J_EyeMed_CMS_837_DBLoad_ODS</t>
         </is>
       </c>
       <c r="B54" t="inlineStr"/>
       <c r="C54" t="inlineStr">
         <is>
-          <t>tFTPPut</t>
+          <t>tMap</t>
         </is>
       </c>
       <c r="D54" t="inlineStr"/>
@@ -2233,13 +1726,13 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>SC_AS400_To_DropZone_MD</t>
+          <t>J_EyeMed_CMS_837_DBLoad_ODS</t>
         </is>
       </c>
       <c r="B55" t="inlineStr"/>
       <c r="C55" t="inlineStr">
         <is>
-          <t>tAS400Input</t>
+          <t>tFlowToIterate</t>
         </is>
       </c>
       <c r="D55" t="inlineStr"/>
@@ -2247,13 +1740,13 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>SC_AS400_To_DropZone_MD</t>
+          <t>J_EyeMed_CMS_837_DBLoad_ODS</t>
         </is>
       </c>
       <c r="B56" t="inlineStr"/>
       <c r="C56" t="inlineStr">
         <is>
-          <t>tFileOutputDelimited</t>
+          <t>tJavaRow</t>
         </is>
       </c>
       <c r="D56" t="inlineStr"/>
@@ -2261,13 +1754,13 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>SC_AS400_To_DropZone_MD</t>
+          <t>J_EyeMed_CMS_837_DBLoad_ODS</t>
         </is>
       </c>
       <c r="B57" t="inlineStr"/>
       <c r="C57" t="inlineStr">
         <is>
-          <t>tFTPConnection</t>
+          <t>tMSSqlOutput</t>
         </is>
       </c>
       <c r="D57" t="inlineStr"/>
@@ -2275,13 +1768,13 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>SC_AS400_To_DropZone_MD</t>
+          <t>J_EyeMed_CMS_837_DBLoad_ODS</t>
         </is>
       </c>
       <c r="B58" t="inlineStr"/>
       <c r="C58" t="inlineStr">
         <is>
-          <t>tPrejob</t>
+          <t>tSendMail</t>
         </is>
       </c>
       <c r="D58" t="inlineStr"/>
@@ -2289,13 +1782,13 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>SC_AS400_To_DropZone_MD</t>
+          <t>J_EyeMed_CMS_837_DBLoad_ODS</t>
         </is>
       </c>
       <c r="B59" t="inlineStr"/>
       <c r="C59" t="inlineStr">
         <is>
-          <t>tJava</t>
+          <t>tLogCatcher</t>
         </is>
       </c>
       <c r="D59" t="inlineStr"/>
@@ -2303,13 +1796,13 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>SC_AS400_To_DropZone_MD</t>
+          <t>J_EyeMed_CMS_837_DBLoad_ODS</t>
         </is>
       </c>
       <c r="B60" t="inlineStr"/>
       <c r="C60" t="inlineStr">
         <is>
-          <t>tLibraryLoad</t>
+          <t>tMap</t>
         </is>
       </c>
       <c r="D60" t="inlineStr"/>
@@ -2317,13 +1810,13 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>SC_AS400_To_DropZone_MD</t>
+          <t>J_EyeMed_CMS_837_DBLoad_ODS</t>
         </is>
       </c>
       <c r="B61" t="inlineStr"/>
       <c r="C61" t="inlineStr">
         <is>
-          <t>tJava</t>
+          <t>tFlowToIterate</t>
         </is>
       </c>
       <c r="D61" t="inlineStr"/>
@@ -2331,13 +1824,13 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>SC_AS400_To_DropZone_MD</t>
+          <t>J_EyeMed_CMS_837_DBLoad_ODS</t>
         </is>
       </c>
       <c r="B62" t="inlineStr"/>
       <c r="C62" t="inlineStr">
         <is>
-          <t>tFileDelete</t>
+          <t>tMSSqlOutput</t>
         </is>
       </c>
       <c r="D62" t="inlineStr"/>
@@ -2345,13 +1838,13 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>SC_AS400_To_DropZone_MD</t>
+          <t>J_EyeMed_CMS_837_DBLoad_ODS</t>
         </is>
       </c>
       <c r="B63" t="inlineStr"/>
       <c r="C63" t="inlineStr">
         <is>
-          <t>tJava</t>
+          <t>tSendMail</t>
         </is>
       </c>
       <c r="D63" t="inlineStr"/>
@@ -2359,13 +1852,13 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>SC_AS400_To_DropZone_MD</t>
+          <t>J_EyeMed_CMS_837_DBLoad_ODS</t>
         </is>
       </c>
       <c r="B64" t="inlineStr"/>
       <c r="C64" t="inlineStr">
         <is>
-          <t>tAS400Connection</t>
+          <t>tDie</t>
         </is>
       </c>
       <c r="D64" t="inlineStr"/>
@@ -2373,13 +1866,13 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>SC_AS400_To_DropZone_MD</t>
+          <t>J_EyeMed_CMS_837_DBLoad_ODS</t>
         </is>
       </c>
       <c r="B65" t="inlineStr"/>
       <c r="C65" t="inlineStr">
         <is>
-          <t>Implicit_context_joblet</t>
+          <t>tFTPDelete</t>
         </is>
       </c>
       <c r="D65" t="inlineStr"/>
@@ -2387,13 +1880,13 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>SC_AS400_To_DropZone_MD</t>
+          <t>J_EyeMed_CMS_837_DBLoad_ODS</t>
         </is>
       </c>
       <c r="B66" t="inlineStr"/>
       <c r="C66" t="inlineStr">
         <is>
-          <t>Job_Start</t>
+          <t>tFileInputXML</t>
         </is>
       </c>
       <c r="D66" t="inlineStr"/>
@@ -2401,13 +1894,13 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>SC_AS400_To_DropZone_MD</t>
+          <t>J_EyeMed_CMS_837_DBLoad_ODS</t>
         </is>
       </c>
       <c r="B67" t="inlineStr"/>
       <c r="C67" t="inlineStr">
         <is>
-          <t>tMysqlConnection</t>
+          <t>tMap</t>
         </is>
       </c>
       <c r="D67" t="inlineStr"/>
@@ -2415,13 +1908,13 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>SC_AS400_To_DropZone_MD</t>
+          <t>J_EyeMed_CMS_837_DBLoad_ODS</t>
         </is>
       </c>
       <c r="B68" t="inlineStr"/>
       <c r="C68" t="inlineStr">
         <is>
-          <t>tFixedFlowInput</t>
+          <t>tHashOutput</t>
         </is>
       </c>
       <c r="D68" t="inlineStr"/>
@@ -2429,13 +1922,13 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>SC_AS400_To_DropZone_MD</t>
+          <t>J_EyeMed_CMS_837_DBLoad_ODS</t>
         </is>
       </c>
       <c r="B69" t="inlineStr"/>
       <c r="C69" t="inlineStr">
         <is>
-          <t>tLogRow</t>
+          <t>tPostjob</t>
         </is>
       </c>
       <c r="D69" t="inlineStr"/>
@@ -2443,13 +1936,13 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>SC_AS400_To_DropZone_MD</t>
+          <t>J_EyeMed_CMS_837_DBLoad_ODS</t>
         </is>
       </c>
       <c r="B70" t="inlineStr"/>
       <c r="C70" t="inlineStr">
         <is>
-          <t>tMysqlOutput</t>
+          <t>tMSSqlClose</t>
         </is>
       </c>
       <c r="D70" t="inlineStr"/>
@@ -2457,13 +1950,13 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>SC_AS400_To_DropZone_MD</t>
+          <t>J_EyeMed_CMS_837_DBLoad_ODS</t>
         </is>
       </c>
       <c r="B71" t="inlineStr"/>
       <c r="C71" t="inlineStr">
         <is>
-          <t>Job_End</t>
+          <t>tFixedFlowInput</t>
         </is>
       </c>
       <c r="D71" t="inlineStr"/>
@@ -2471,13 +1964,13 @@
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>SC_AS400_To_DropZone_MD</t>
+          <t>J_EyeMed_CMS_837_DBLoad_ODS</t>
         </is>
       </c>
       <c r="B72" t="inlineStr"/>
       <c r="C72" t="inlineStr">
         <is>
-          <t>tMysqlInput</t>
+          <t>tHashOutput</t>
         </is>
       </c>
       <c r="D72" t="inlineStr"/>
@@ -2485,13 +1978,13 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>SC_AS400_To_DropZone_MD</t>
+          <t>J_EyeMed_CMS_837_DBLoad_ODS</t>
         </is>
       </c>
       <c r="B73" t="inlineStr"/>
       <c r="C73" t="inlineStr">
         <is>
-          <t>tJavaRow</t>
+          <t>tFileCopy</t>
         </is>
       </c>
       <c r="D73" t="inlineStr"/>
@@ -2499,13 +1992,13 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>SC_AS400_To_DropZone_MD</t>
+          <t>J_EyeMed_CMS_837_DBLoad_ODS</t>
         </is>
       </c>
       <c r="B74" t="inlineStr"/>
       <c r="C74" t="inlineStr">
         <is>
-          <t>tDie</t>
+          <t>tJava</t>
         </is>
       </c>
       <c r="D74" t="inlineStr"/>
@@ -2513,13 +2006,13 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>SC_AS400_To_DropZone_MD</t>
+          <t>J_EyeMed_CMS_837_DBLoad_ODS</t>
         </is>
       </c>
       <c r="B75" t="inlineStr"/>
       <c r="C75" t="inlineStr">
         <is>
-          <t>tDie</t>
+          <t>tFileList</t>
         </is>
       </c>
       <c r="D75" t="inlineStr"/>
@@ -2527,13 +2020,13 @@
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>SC_AS400_To_DropZone_MD</t>
+          <t>J_EyeMed_CMS_837_DBLoad_ODS</t>
         </is>
       </c>
       <c r="B76" t="inlineStr"/>
       <c r="C76" t="inlineStr">
         <is>
-          <t>tDie</t>
+          <t>tFileCopy</t>
         </is>
       </c>
       <c r="D76" t="inlineStr"/>
@@ -2541,13 +2034,13 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>SC_AS400_To_DropZone_MD</t>
+          <t>J_EyeMed_CMS_837_DBLoad_ODS</t>
         </is>
       </c>
       <c r="B77" t="inlineStr"/>
       <c r="C77" t="inlineStr">
         <is>
-          <t>tLibraryLoad</t>
+          <t>tJava</t>
         </is>
       </c>
       <c r="D77" t="inlineStr"/>
@@ -2555,13 +2048,13 @@
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>SC_AS400_To_DropZone_MD</t>
+          <t>J_EyeMed_CMS_837_DBLoad_ODS</t>
         </is>
       </c>
       <c r="B78" t="inlineStr"/>
       <c r="C78" t="inlineStr">
         <is>
-          <t>tMysqlInput</t>
+          <t>tMSSqlConnection</t>
         </is>
       </c>
       <c r="D78" t="inlineStr"/>
@@ -2569,13 +2062,13 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>SC_AS400_To_DropZone_MD</t>
+          <t>J_EyeMed_CMS_837_DBLoad_ODS</t>
         </is>
       </c>
       <c r="B79" t="inlineStr"/>
       <c r="C79" t="inlineStr">
         <is>
-          <t>tFlowToIterate</t>
+          <t>tFileList</t>
         </is>
       </c>
       <c r="D79" t="inlineStr"/>
@@ -2583,13 +2076,13 @@
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>SC_AS400_To_DropZone_MD</t>
+          <t>J_EyeMed_CMS_837_DBLoad_ODS</t>
         </is>
       </c>
       <c r="B80" t="inlineStr"/>
       <c r="C80" t="inlineStr">
         <is>
-          <t>tMysqlInput</t>
+          <t>tFileInputRaw</t>
         </is>
       </c>
       <c r="D80" t="inlineStr"/>
@@ -2597,13 +2090,13 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>SC_AS400_To_DropZone_MD</t>
+          <t>J_EyeMed_CMS_837_DBLoad_ODS</t>
         </is>
       </c>
       <c r="B81" t="inlineStr"/>
       <c r="C81" t="inlineStr">
         <is>
-          <t>tJavaRow</t>
+          <t>tHMap</t>
         </is>
       </c>
       <c r="D81" t="inlineStr"/>
@@ -2611,13 +2104,13 @@
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>SC_AS400_To_DropZone_MD</t>
+          <t>J_EyeMed_CMS_837_DBLoad_ODS</t>
         </is>
       </c>
       <c r="B82" t="inlineStr"/>
       <c r="C82" t="inlineStr">
         <is>
-          <t>tDie</t>
+          <t>tFileOutputRaw</t>
         </is>
       </c>
       <c r="D82" t="inlineStr"/>
@@ -2625,13 +2118,13 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>SC_AS400_To_DropZone_MD</t>
+          <t>J_EyeMed_CMS_837_DBLoad_ODS</t>
         </is>
       </c>
       <c r="B83" t="inlineStr"/>
       <c r="C83" t="inlineStr">
         <is>
-          <t>tJava</t>
+          <t>tDie</t>
         </is>
       </c>
       <c r="D83" t="inlineStr"/>
@@ -2639,13 +2132,13 @@
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>SC_AS400_To_DropZone_MD</t>
+          <t>J_EyeMed_CMS_837_DBLoad_ODS</t>
         </is>
       </c>
       <c r="B84" t="inlineStr"/>
       <c r="C84" t="inlineStr">
         <is>
-          <t>tPostjob</t>
+          <t>tFileList</t>
         </is>
       </c>
       <c r="D84" t="inlineStr"/>
@@ -2653,13 +2146,13 @@
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>SC_AS400_To_DropZone_MD</t>
+          <t>J_EyeMed_CMS_837_DBLoad_ODS</t>
         </is>
       </c>
       <c r="B85" t="inlineStr"/>
       <c r="C85" t="inlineStr">
         <is>
-          <t>tAS400Close</t>
+          <t>tJava</t>
         </is>
       </c>
       <c r="D85" t="inlineStr"/>
@@ -2667,13 +2160,13 @@
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>SC_AS400_To_DropZone_MD</t>
+          <t>J_EyeMed_CMS_837_DBLoad_ODS</t>
         </is>
       </c>
       <c r="B86" t="inlineStr"/>
       <c r="C86" t="inlineStr">
         <is>
-          <t>tMysqlClose</t>
+          <t>tMSSqlInput</t>
         </is>
       </c>
       <c r="D86" t="inlineStr"/>
@@ -2681,13 +2174,13 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>SC_AS400_To_DropZone_MD</t>
+          <t>J_EyeMed_CMS_837_DBLoad_ODS</t>
         </is>
       </c>
       <c r="B87" t="inlineStr"/>
       <c r="C87" t="inlineStr">
         <is>
-          <t>tJava</t>
+          <t>tMap</t>
         </is>
       </c>
       <c r="D87" t="inlineStr"/>
@@ -2695,13 +2188,13 @@
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>SC_AS400_To_DropZone_MD</t>
+          <t>J_EyeMed_CMS_837_DBLoad_ODS</t>
         </is>
       </c>
       <c r="B88" t="inlineStr"/>
       <c r="C88" t="inlineStr">
         <is>
-          <t>tMysqlInput</t>
+          <t>tSetGlobalVar</t>
         </is>
       </c>
       <c r="D88" t="inlineStr"/>
@@ -2709,13 +2202,13 @@
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>SC_AS400_To_DropZone_MD</t>
+          <t>J_EyeMed_CMS_837_DBLoad_ODS</t>
         </is>
       </c>
       <c r="B89" t="inlineStr"/>
       <c r="C89" t="inlineStr">
         <is>
-          <t>tJavaRow</t>
+          <t>tFileInputXML</t>
         </is>
       </c>
       <c r="D89" t="inlineStr"/>
@@ -2723,13 +2216,13 @@
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>SC_AS400_To_DropZone_MD</t>
+          <t>J_EyeMed_CMS_837_DBLoad_ODS</t>
         </is>
       </c>
       <c r="B90" t="inlineStr"/>
       <c r="C90" t="inlineStr">
         <is>
-          <t>tJava</t>
+          <t>tMap</t>
         </is>
       </c>
       <c r="D90" t="inlineStr"/>
@@ -2737,13 +2230,13 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>SC_AS400_To_DropZone_MD</t>
+          <t>J_EyeMed_CMS_837_DBLoad_ODS</t>
         </is>
       </c>
       <c r="B91" t="inlineStr"/>
       <c r="C91" t="inlineStr">
         <is>
-          <t>tFileDelete</t>
+          <t>tMap</t>
         </is>
       </c>
       <c r="D91" t="inlineStr"/>
@@ -2751,13 +2244,13 @@
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>SC_AS400_To_DropZone_MD</t>
+          <t>J_EyeMed_CMS_837_DBLoad_ODS</t>
         </is>
       </c>
       <c r="B92" t="inlineStr"/>
       <c r="C92" t="inlineStr">
         <is>
-          <t>tFixedFlowInput</t>
+          <t>tHashInput</t>
         </is>
       </c>
       <c r="D92" t="inlineStr"/>
@@ -2765,13 +2258,13 @@
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>SC_AS400_To_DropZone_MD</t>
+          <t>J_EyeMed_CMS_837_DBLoad_ODS</t>
         </is>
       </c>
       <c r="B93" t="inlineStr"/>
       <c r="C93" t="inlineStr">
         <is>
-          <t>tLogRow</t>
+          <t>tMSSqlOutput</t>
         </is>
       </c>
       <c r="D93" t="inlineStr"/>
@@ -2779,13 +2272,13 @@
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>SC_AS400_To_DropZone_MD</t>
+          <t>J_EyeMed_CMS_837_DBLoad_ODS</t>
         </is>
       </c>
       <c r="B94" t="inlineStr"/>
       <c r="C94" t="inlineStr">
         <is>
-          <t>tMysqlOutput</t>
+          <t>tFileInputXML</t>
         </is>
       </c>
       <c r="D94" t="inlineStr"/>
@@ -2793,13 +2286,13 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>SC_AS400_To_DropZone_MD</t>
+          <t>J_EyeMed_CMS_837_DBLoad_ODS</t>
         </is>
       </c>
       <c r="B95" t="inlineStr"/>
       <c r="C95" t="inlineStr">
         <is>
-          <t>Job_End</t>
+          <t>tMap</t>
         </is>
       </c>
       <c r="D95" t="inlineStr"/>
@@ -2807,13 +2300,13 @@
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>SC_AS400_To_DropZone_MD</t>
+          <t>J_EyeMed_CMS_837_DBLoad_ODS</t>
         </is>
       </c>
       <c r="B96" t="inlineStr"/>
       <c r="C96" t="inlineStr">
         <is>
-          <t>tFTPClose</t>
+          <t>tMap</t>
         </is>
       </c>
       <c r="D96" t="inlineStr"/>
@@ -2821,13 +2314,13 @@
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>SC_AS400_To_DropZone_MD</t>
+          <t>J_EyeMed_CMS_837_DBLoad_ODS</t>
         </is>
       </c>
       <c r="B97" t="inlineStr"/>
       <c r="C97" t="inlineStr">
         <is>
-          <t>Job_Error</t>
+          <t>tHashInput</t>
         </is>
       </c>
       <c r="D97" t="inlineStr"/>
@@ -2835,13 +2328,13 @@
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>SC_AS400_To_DropZone_MD</t>
+          <t>J_EyeMed_CMS_837_DBLoad_ODS</t>
         </is>
       </c>
       <c r="B98" t="inlineStr"/>
       <c r="C98" t="inlineStr">
         <is>
-          <t>tMysqlInput</t>
+          <t>tMSSqlOutput</t>
         </is>
       </c>
       <c r="D98" t="inlineStr"/>
@@ -2849,13 +2342,13 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>SC_AS400_To_DropZone_MD</t>
+          <t>J_EyeMed_CMS_837_DBLoad_ODS</t>
         </is>
       </c>
       <c r="B99" t="inlineStr"/>
       <c r="C99" t="inlineStr">
         <is>
-          <t>tFlowToIterate</t>
+          <t>tFileInputXML</t>
         </is>
       </c>
       <c r="D99" t="inlineStr"/>
@@ -2863,13 +2356,13 @@
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>SC_AS400_To_DropZone_MD</t>
+          <t>J_EyeMed_CMS_837_DBLoad_ODS</t>
         </is>
       </c>
       <c r="B100" t="inlineStr"/>
       <c r="C100" t="inlineStr">
         <is>
-          <t>tJava</t>
+          <t>tMap</t>
         </is>
       </c>
       <c r="D100" t="inlineStr"/>
@@ -2877,13 +2370,13 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>SC_AS400_To_DropZone_MD</t>
+          <t>J_EyeMed_CMS_837_DBLoad_ODS</t>
         </is>
       </c>
       <c r="B101" t="inlineStr"/>
       <c r="C101" t="inlineStr">
         <is>
-          <t>tJava</t>
+          <t>tMap</t>
         </is>
       </c>
       <c r="D101" t="inlineStr"/>
@@ -2891,13 +2384,13 @@
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>SC_AS400_To_DropZone_MD</t>
+          <t>J_EyeMed_CMS_837_DBLoad_ODS</t>
         </is>
       </c>
       <c r="B102" t="inlineStr"/>
       <c r="C102" t="inlineStr">
         <is>
-          <t>tFTPPut</t>
+          <t>tHashInput</t>
         </is>
       </c>
       <c r="D102" t="inlineStr"/>
@@ -2905,13 +2398,13 @@
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>SC_AS400_To_DropZone_MD</t>
+          <t>J_EyeMed_CMS_837_DBLoad_ODS</t>
         </is>
       </c>
       <c r="B103" t="inlineStr"/>
       <c r="C103" t="inlineStr">
         <is>
-          <t>tAS400Input</t>
+          <t>tMSSqlOutput</t>
         </is>
       </c>
       <c r="D103" t="inlineStr"/>
@@ -2919,13 +2412,13 @@
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>SC_AS400_To_DropZone_MD</t>
+          <t>J_EyeMed_CMS_837_DBLoad_ODS</t>
         </is>
       </c>
       <c r="B104" t="inlineStr"/>
       <c r="C104" t="inlineStr">
         <is>
-          <t>tFileOutputDelimited</t>
+          <t>tFixedFlowInput</t>
         </is>
       </c>
       <c r="D104" t="inlineStr"/>
@@ -2933,13 +2426,13 @@
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>SC_AS400_To_DropZone_MD</t>
+          <t>J_EyeMed_CMS_837_DBLoad_ODS</t>
         </is>
       </c>
       <c r="B105" t="inlineStr"/>
       <c r="C105" t="inlineStr">
         <is>
-          <t>tFTPConnection</t>
+          <t>tJavaRow</t>
         </is>
       </c>
       <c r="D105" t="inlineStr"/>
@@ -2947,13 +2440,13 @@
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>SC_AS400_To_DropZone_MD</t>
+          <t>J_EyeMed_CMS_837_DBLoad_ODS</t>
         </is>
       </c>
       <c r="B106" t="inlineStr"/>
       <c r="C106" t="inlineStr">
         <is>
-          <t>tPrejob</t>
+          <t>tFileList</t>
         </is>
       </c>
       <c r="D106" t="inlineStr"/>
@@ -2961,13 +2454,13 @@
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>SC_AS400_To_DropZone_MD</t>
+          <t>J_EyeMed_CMS_837_DBLoad_ODS</t>
         </is>
       </c>
       <c r="B107" t="inlineStr"/>
       <c r="C107" t="inlineStr">
         <is>
-          <t>tJava</t>
+          <t>tFileCopy</t>
         </is>
       </c>
       <c r="D107" t="inlineStr"/>
@@ -2975,13 +2468,13 @@
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>SC_AS400_To_DropZone_MD</t>
+          <t>J_EyeMed_CMS_837_DBLoad_ODS</t>
         </is>
       </c>
       <c r="B108" t="inlineStr"/>
       <c r="C108" t="inlineStr">
         <is>
-          <t>tLibraryLoad</t>
+          <t>tJava</t>
         </is>
       </c>
       <c r="D108" t="inlineStr"/>
@@ -2989,13 +2482,13 @@
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>SC_AS400_To_DropZone_MD</t>
+          <t>J_EyeMed_CMS_837_DBLoad_ODS</t>
         </is>
       </c>
       <c r="B109" t="inlineStr"/>
       <c r="C109" t="inlineStr">
         <is>
-          <t>tJava</t>
+          <t>tSendMail</t>
         </is>
       </c>
       <c r="D109" t="inlineStr"/>
@@ -3003,13 +2496,13 @@
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>SC_AS400_To_DropZone_MD</t>
+          <t>J_EyeMed_CMS_837_DBLoad_ODS</t>
         </is>
       </c>
       <c r="B110" t="inlineStr"/>
       <c r="C110" t="inlineStr">
         <is>
-          <t>tFileDelete</t>
+          <t>tFileInputXML</t>
         </is>
       </c>
       <c r="D110" t="inlineStr"/>
@@ -3017,13 +2510,13 @@
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>SC_AS400_To_DropZone_MD</t>
+          <t>J_EyeMed_CMS_837_DBLoad_ODS</t>
         </is>
       </c>
       <c r="B111" t="inlineStr"/>
       <c r="C111" t="inlineStr">
         <is>
-          <t>tJava</t>
+          <t>tMap</t>
         </is>
       </c>
       <c r="D111" t="inlineStr"/>
@@ -3031,13 +2524,13 @@
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>SC_AS400_To_DropZone_MD</t>
+          <t>J_EyeMed_CMS_837_DBLoad_ODS</t>
         </is>
       </c>
       <c r="B112" t="inlineStr"/>
       <c r="C112" t="inlineStr">
         <is>
-          <t>tAS400Connection</t>
+          <t>tMap</t>
         </is>
       </c>
       <c r="D112" t="inlineStr"/>
@@ -3045,13 +2538,13 @@
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>SC_AS400_To_DropZone_MD</t>
+          <t>J_EyeMed_CMS_837_DBLoad_ODS</t>
         </is>
       </c>
       <c r="B113" t="inlineStr"/>
       <c r="C113" t="inlineStr">
         <is>
-          <t>Implicit_context_joblet</t>
+          <t>tMSSqlOutput</t>
         </is>
       </c>
       <c r="D113" t="inlineStr"/>
@@ -3059,13 +2552,13 @@
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>SC_AS400_To_DropZone_MD</t>
+          <t>J_EyeMed_CMS_837_DBLoad_ODS</t>
         </is>
       </c>
       <c r="B114" t="inlineStr"/>
       <c r="C114" t="inlineStr">
         <is>
-          <t>Job_Start</t>
+          <t>tFileInputDelimited</t>
         </is>
       </c>
       <c r="D114" t="inlineStr"/>
@@ -3073,13 +2566,13 @@
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>SC_AS400_To_DropZone_MD</t>
+          <t>J_EyeMed_CMS_837_DBLoad_ODS</t>
         </is>
       </c>
       <c r="B115" t="inlineStr"/>
       <c r="C115" t="inlineStr">
         <is>
-          <t>tMysqlConnection</t>
+          <t>tJavaRow</t>
         </is>
       </c>
       <c r="D115" t="inlineStr"/>
@@ -3087,13 +2580,13 @@
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>SC_AS400_To_DropZone_MD</t>
+          <t>J_EyeMed_CMS_837_DBLoad_ODS</t>
         </is>
       </c>
       <c r="B116" t="inlineStr"/>
       <c r="C116" t="inlineStr">
         <is>
-          <t>tFixedFlowInput</t>
+          <t>tFileInputXML</t>
         </is>
       </c>
       <c r="D116" t="inlineStr"/>
@@ -3101,13 +2594,13 @@
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t>SC_AS400_To_DropZone_MD</t>
+          <t>J_EyeMed_CMS_837_DBLoad_ODS</t>
         </is>
       </c>
       <c r="B117" t="inlineStr"/>
       <c r="C117" t="inlineStr">
         <is>
-          <t>tLogRow</t>
+          <t>tMap</t>
         </is>
       </c>
       <c r="D117" t="inlineStr"/>
@@ -3115,13 +2608,13 @@
     <row r="118">
       <c r="A118" t="inlineStr">
         <is>
-          <t>SC_AS400_To_DropZone_MD</t>
+          <t>J_EyeMed_CMS_837_DBLoad_ODS</t>
         </is>
       </c>
       <c r="B118" t="inlineStr"/>
       <c r="C118" t="inlineStr">
         <is>
-          <t>tMysqlOutput</t>
+          <t>tMap</t>
         </is>
       </c>
       <c r="D118" t="inlineStr"/>
@@ -3129,13 +2622,13 @@
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
-          <t>SC_AS400_To_DropZone_MD</t>
+          <t>J_EyeMed_CMS_837_DBLoad_ODS</t>
         </is>
       </c>
       <c r="B119" t="inlineStr"/>
       <c r="C119" t="inlineStr">
         <is>
-          <t>Job_End</t>
+          <t>tMSSqlInput</t>
         </is>
       </c>
       <c r="D119" t="inlineStr"/>
@@ -3143,13 +2636,13 @@
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>SC_AS400_To_DropZone_MD</t>
+          <t>J_EyeMed_CMS_837_DBLoad_ODS</t>
         </is>
       </c>
       <c r="B120" t="inlineStr"/>
       <c r="C120" t="inlineStr">
         <is>
-          <t>tMysqlInput</t>
+          <t>tMSSqlOutput</t>
         </is>
       </c>
       <c r="D120" t="inlineStr"/>
@@ -3157,13 +2650,13 @@
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>SC_AS400_To_DropZone_MD</t>
+          <t>J_EyeMed_CMS_837_DBLoad_ODS</t>
         </is>
       </c>
       <c r="B121" t="inlineStr"/>
       <c r="C121" t="inlineStr">
         <is>
-          <t>tJavaRow</t>
+          <t>tFTPConnection</t>
         </is>
       </c>
       <c r="D121" t="inlineStr"/>
@@ -3171,13 +2664,13 @@
     <row r="122">
       <c r="A122" t="inlineStr">
         <is>
-          <t>SC_AS400_To_DropZone_MD</t>
+          <t>J_EyeMed_CMS_837_DBLoad_ODS</t>
         </is>
       </c>
       <c r="B122" t="inlineStr"/>
       <c r="C122" t="inlineStr">
         <is>
-          <t>tDie</t>
+          <t>tFTPFileList</t>
         </is>
       </c>
       <c r="D122" t="inlineStr"/>
@@ -3185,13 +2678,13 @@
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
-          <t>SC_AS400_To_DropZone_MD</t>
+          <t>J_EyeMed_CMS_837_DBLoad_ODS</t>
         </is>
       </c>
       <c r="B123" t="inlineStr"/>
       <c r="C123" t="inlineStr">
         <is>
-          <t>tDie</t>
+          <t>tFTPGet</t>
         </is>
       </c>
       <c r="D123" t="inlineStr"/>
@@ -3199,13 +2692,13 @@
     <row r="124">
       <c r="A124" t="inlineStr">
         <is>
-          <t>SC_AS400_To_DropZone_MD</t>
+          <t>J_EyeMed_CMS_837_DBLoad_ODS</t>
         </is>
       </c>
       <c r="B124" t="inlineStr"/>
       <c r="C124" t="inlineStr">
         <is>
-          <t>tDie</t>
+          <t>tSendMail</t>
         </is>
       </c>
       <c r="D124" t="inlineStr"/>
@@ -3213,13 +2706,13 @@
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>SC_AS400_To_DropZone_MD</t>
+          <t>J_EyeMed_CMS_837_DBLoad_ODS</t>
         </is>
       </c>
       <c r="B125" t="inlineStr"/>
       <c r="C125" t="inlineStr">
         <is>
-          <t>tLibraryLoad</t>
+          <t>tSendMail</t>
         </is>
       </c>
       <c r="D125" t="inlineStr"/>
@@ -3227,13 +2720,13 @@
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>SC_AS400_To_DropZone_MD</t>
+          <t>J_EyeMed_CMS_837_DBLoad_ODS</t>
         </is>
       </c>
       <c r="B126" t="inlineStr"/>
       <c r="C126" t="inlineStr">
         <is>
-          <t>tMysqlInput</t>
+          <t>tDie</t>
         </is>
       </c>
       <c r="D126" t="inlineStr"/>
@@ -3241,13 +2734,13 @@
     <row r="127">
       <c r="A127" t="inlineStr">
         <is>
-          <t>SC_AS400_To_DropZone_MD</t>
+          <t>J_EyeMed_CMS_837_DBLoad_ODS</t>
         </is>
       </c>
       <c r="B127" t="inlineStr"/>
       <c r="C127" t="inlineStr">
         <is>
-          <t>tFlowToIterate</t>
+          <t>tPrejob</t>
         </is>
       </c>
       <c r="D127" t="inlineStr"/>
@@ -3255,13 +2748,13 @@
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
-          <t>SC_AS400_To_DropZone_MD</t>
+          <t>J_EyeMed_CMS_837_DBLoad_ODS</t>
         </is>
       </c>
       <c r="B128" t="inlineStr"/>
       <c r="C128" t="inlineStr">
         <is>
-          <t>tMysqlInput</t>
+          <t>tMSSqlConnection</t>
         </is>
       </c>
       <c r="D128" t="inlineStr"/>
@@ -3269,13 +2762,13 @@
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t>SC_AS400_To_DropZone_MD</t>
+          <t>J_EyeMed_CMS_837_DBLoad_ODS</t>
         </is>
       </c>
       <c r="B129" t="inlineStr"/>
       <c r="C129" t="inlineStr">
         <is>
-          <t>tJavaRow</t>
+          <t>tStatCatcher</t>
         </is>
       </c>
       <c r="D129" t="inlineStr"/>
@@ -3283,13 +2776,13 @@
     <row r="130">
       <c r="A130" t="inlineStr">
         <is>
-          <t>SC_AS400_To_DropZone_MD</t>
+          <t>J_EyeMed_CMS_837_DBLoad_ODS</t>
         </is>
       </c>
       <c r="B130" t="inlineStr"/>
       <c r="C130" t="inlineStr">
         <is>
-          <t>tDie</t>
+          <t>tMap</t>
         </is>
       </c>
       <c r="D130" t="inlineStr"/>
@@ -3297,13 +2790,13 @@
     <row r="131">
       <c r="A131" t="inlineStr">
         <is>
-          <t>SC_AS400_To_DropZone_MD</t>
+          <t>J_EyeMed_CMS_837_DBLoad_ODS</t>
         </is>
       </c>
       <c r="B131" t="inlineStr"/>
       <c r="C131" t="inlineStr">
         <is>
-          <t>tJava</t>
+          <t>tFlowToIterate</t>
         </is>
       </c>
       <c r="D131" t="inlineStr"/>
@@ -3311,13 +2804,13 @@
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>SC_AS400_To_DropZone_MD</t>
+          <t>J_EyeMed_CMS_837_DBLoad_ODS</t>
         </is>
       </c>
       <c r="B132" t="inlineStr"/>
       <c r="C132" t="inlineStr">
         <is>
-          <t>tPostjob</t>
+          <t>tJavaRow</t>
         </is>
       </c>
       <c r="D132" t="inlineStr"/>
@@ -3325,13 +2818,13 @@
     <row r="133">
       <c r="A133" t="inlineStr">
         <is>
-          <t>SC_AS400_To_DropZone_MD</t>
+          <t>J_EyeMed_CMS_837_DBLoad_ODS</t>
         </is>
       </c>
       <c r="B133" t="inlineStr"/>
       <c r="C133" t="inlineStr">
         <is>
-          <t>tAS400Close</t>
+          <t>tMSSqlOutput</t>
         </is>
       </c>
       <c r="D133" t="inlineStr"/>
@@ -3339,13 +2832,13 @@
     <row r="134">
       <c r="A134" t="inlineStr">
         <is>
-          <t>SC_AS400_To_DropZone_MD</t>
+          <t>J_EyeMed_CMS_837_DBLoad_ODS</t>
         </is>
       </c>
       <c r="B134" t="inlineStr"/>
       <c r="C134" t="inlineStr">
         <is>
-          <t>tMysqlClose</t>
+          <t>tSendMail</t>
         </is>
       </c>
       <c r="D134" t="inlineStr"/>
@@ -3353,13 +2846,13 @@
     <row r="135">
       <c r="A135" t="inlineStr">
         <is>
-          <t>SC_AS400_To_DropZone_MD</t>
+          <t>J_EyeMed_CMS_837_DBLoad_ODS</t>
         </is>
       </c>
       <c r="B135" t="inlineStr"/>
       <c r="C135" t="inlineStr">
         <is>
-          <t>tJava</t>
+          <t>tLogCatcher</t>
         </is>
       </c>
       <c r="D135" t="inlineStr"/>
@@ -3367,13 +2860,13 @@
     <row r="136">
       <c r="A136" t="inlineStr">
         <is>
-          <t>SC_AS400_To_DropZone_MD</t>
+          <t>J_EyeMed_CMS_837_DBLoad_ODS</t>
         </is>
       </c>
       <c r="B136" t="inlineStr"/>
       <c r="C136" t="inlineStr">
         <is>
-          <t>tMysqlInput</t>
+          <t>tMap</t>
         </is>
       </c>
       <c r="D136" t="inlineStr"/>
@@ -3381,13 +2874,13 @@
     <row r="137">
       <c r="A137" t="inlineStr">
         <is>
-          <t>SC_AS400_To_DropZone_MD</t>
+          <t>J_EyeMed_CMS_837_DBLoad_ODS</t>
         </is>
       </c>
       <c r="B137" t="inlineStr"/>
       <c r="C137" t="inlineStr">
         <is>
-          <t>tJavaRow</t>
+          <t>tFlowToIterate</t>
         </is>
       </c>
       <c r="D137" t="inlineStr"/>
@@ -3395,13 +2888,13 @@
     <row r="138">
       <c r="A138" t="inlineStr">
         <is>
-          <t>SC_AS400_To_DropZone_MD</t>
+          <t>J_EyeMed_CMS_837_DBLoad_ODS</t>
         </is>
       </c>
       <c r="B138" t="inlineStr"/>
       <c r="C138" t="inlineStr">
         <is>
-          <t>tJava</t>
+          <t>tMSSqlOutput</t>
         </is>
       </c>
       <c r="D138" t="inlineStr"/>
@@ -3409,13 +2902,13 @@
     <row r="139">
       <c r="A139" t="inlineStr">
         <is>
-          <t>SC_AS400_To_DropZone_MD</t>
+          <t>J_EyeMed_CMS_837_DBLoad_ODS</t>
         </is>
       </c>
       <c r="B139" t="inlineStr"/>
       <c r="C139" t="inlineStr">
         <is>
-          <t>tFileDelete</t>
+          <t>tSendMail</t>
         </is>
       </c>
       <c r="D139" t="inlineStr"/>
@@ -3423,13 +2916,13 @@
     <row r="140">
       <c r="A140" t="inlineStr">
         <is>
-          <t>SC_AS400_To_DropZone_MD</t>
+          <t>J_EyeMed_CMS_837_DBLoad_ODS</t>
         </is>
       </c>
       <c r="B140" t="inlineStr"/>
       <c r="C140" t="inlineStr">
         <is>
-          <t>tFixedFlowInput</t>
+          <t>tDie</t>
         </is>
       </c>
       <c r="D140" t="inlineStr"/>
@@ -3437,13 +2930,13 @@
     <row r="141">
       <c r="A141" t="inlineStr">
         <is>
-          <t>SC_AS400_To_DropZone_MD</t>
+          <t>J_EyeMed_CMS_837_DBLoad_ODS</t>
         </is>
       </c>
       <c r="B141" t="inlineStr"/>
       <c r="C141" t="inlineStr">
         <is>
-          <t>tLogRow</t>
+          <t>tFTPDelete</t>
         </is>
       </c>
       <c r="D141" t="inlineStr"/>
@@ -3451,13 +2944,13 @@
     <row r="142">
       <c r="A142" t="inlineStr">
         <is>
-          <t>SC_AS400_To_DropZone_MD</t>
+          <t>J_EyeMed_CMS_837_DBLoad_ODS</t>
         </is>
       </c>
       <c r="B142" t="inlineStr"/>
       <c r="C142" t="inlineStr">
         <is>
-          <t>tMysqlOutput</t>
+          <t>tFileInputXML</t>
         </is>
       </c>
       <c r="D142" t="inlineStr"/>
@@ -3465,13 +2958,13 @@
     <row r="143">
       <c r="A143" t="inlineStr">
         <is>
-          <t>SC_AS400_To_DropZone_MD</t>
+          <t>J_EyeMed_CMS_837_DBLoad_ODS</t>
         </is>
       </c>
       <c r="B143" t="inlineStr"/>
       <c r="C143" t="inlineStr">
         <is>
-          <t>Job_End</t>
+          <t>tMap</t>
         </is>
       </c>
       <c r="D143" t="inlineStr"/>
@@ -3479,13 +2972,13 @@
     <row r="144">
       <c r="A144" t="inlineStr">
         <is>
-          <t>SC_AS400_To_DropZone_MD</t>
+          <t>J_EyeMed_CMS_837_DBLoad_ODS</t>
         </is>
       </c>
       <c r="B144" t="inlineStr"/>
       <c r="C144" t="inlineStr">
         <is>
-          <t>tFTPClose</t>
+          <t>tHashOutput</t>
         </is>
       </c>
       <c r="D144" t="inlineStr"/>
@@ -3493,13 +2986,13 @@
     <row r="145">
       <c r="A145" t="inlineStr">
         <is>
-          <t>SC_AS400_To_DropZone_MD</t>
+          <t>J_EyeMed_CMS_837_DBLoad_ODS</t>
         </is>
       </c>
       <c r="B145" t="inlineStr"/>
       <c r="C145" t="inlineStr">
         <is>
-          <t>Job_Error</t>
+          <t>tPostjob</t>
         </is>
       </c>
       <c r="D145" t="inlineStr"/>
@@ -3507,13 +3000,13 @@
     <row r="146">
       <c r="A146" t="inlineStr">
         <is>
-          <t>SC_AS400_To_DropZone_MD</t>
+          <t>J_EyeMed_CMS_837_DBLoad_ODS</t>
         </is>
       </c>
       <c r="B146" t="inlineStr"/>
       <c r="C146" t="inlineStr">
         <is>
-          <t>tMysqlInput</t>
+          <t>tMSSqlClose</t>
         </is>
       </c>
       <c r="D146" t="inlineStr"/>
@@ -3521,13 +3014,13 @@
     <row r="147">
       <c r="A147" t="inlineStr">
         <is>
-          <t>SC_AS400_To_DropZone_MD</t>
+          <t>J_EyeMed_CMS_837_DBLoad_ODS</t>
         </is>
       </c>
       <c r="B147" t="inlineStr"/>
       <c r="C147" t="inlineStr">
         <is>
-          <t>tJavaRow</t>
+          <t>tFixedFlowInput</t>
         </is>
       </c>
       <c r="D147" t="inlineStr"/>
@@ -3535,13 +3028,13 @@
     <row r="148">
       <c r="A148" t="inlineStr">
         <is>
-          <t>SC_AS400_To_DropZone_MD</t>
+          <t>J_EyeMed_CMS_837_DBLoad_ODS</t>
         </is>
       </c>
       <c r="B148" t="inlineStr"/>
       <c r="C148" t="inlineStr">
         <is>
-          <t>tAS400Input</t>
+          <t>tHashOutput</t>
         </is>
       </c>
       <c r="D148" t="inlineStr"/>
@@ -3549,13 +3042,13 @@
     <row r="149">
       <c r="A149" t="inlineStr">
         <is>
-          <t>SC_AS400_To_DropZone_MD</t>
+          <t>J_EyeMed_CMS_837_DBLoad_ODS</t>
         </is>
       </c>
       <c r="B149" t="inlineStr"/>
       <c r="C149" t="inlineStr">
         <is>
-          <t>tDie</t>
+          <t>tFileCopy</t>
         </is>
       </c>
       <c r="D149" t="inlineStr"/>
@@ -3563,13 +3056,13 @@
     <row r="150">
       <c r="A150" t="inlineStr">
         <is>
-          <t>SC_AS400_To_DropZone_MD</t>
+          <t>J_EyeMed_CMS_837_DBLoad_ODS</t>
         </is>
       </c>
       <c r="B150" t="inlineStr"/>
       <c r="C150" t="inlineStr">
         <is>
-          <t>tMysqlConnection</t>
+          <t>tJava</t>
         </is>
       </c>
       <c r="D150" t="inlineStr"/>
@@ -3577,13 +3070,13 @@
     <row r="151">
       <c r="A151" t="inlineStr">
         <is>
-          <t>SC_AS400_To_DropZone_MD</t>
+          <t>J_EyeMed_CMS_837_DBLoad_ODS</t>
         </is>
       </c>
       <c r="B151" t="inlineStr"/>
       <c r="C151" t="inlineStr">
         <is>
-          <t>tDie</t>
+          <t>tFileList</t>
         </is>
       </c>
       <c r="D151" t="inlineStr"/>
@@ -3591,16 +3084,30 @@
     <row r="152">
       <c r="A152" t="inlineStr">
         <is>
-          <t>SC_AS400_To_DropZone_MD</t>
+          <t>J_EyeMed_CMS_837_DBLoad_ODS</t>
         </is>
       </c>
       <c r="B152" t="inlineStr"/>
       <c r="C152" t="inlineStr">
         <is>
-          <t>tMysqlConnection</t>
+          <t>tFileCopy</t>
         </is>
       </c>
       <c r="D152" t="inlineStr"/>
+    </row>
+    <row r="153">
+      <c r="A153" t="inlineStr">
+        <is>
+          <t>J_EyeMed_CMS_837_DBLoad_ODS</t>
+        </is>
+      </c>
+      <c r="B153" t="inlineStr"/>
+      <c r="C153" t="inlineStr">
+        <is>
+          <t>tJava</t>
+        </is>
+      </c>
+      <c r="D153" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -3613,10 +3120,10 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D35"/>
+  <dimension ref="A1:D17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="25" customWidth="1" min="1" max="1"/>
+    <col width="29" customWidth="1" min="1" max="1"/>
     <col width="60" customWidth="1" min="2" max="2"/>
     <col width="10" customWidth="1" min="3" max="3"/>
     <col width="10" customWidth="1" min="4" max="4"/>
@@ -3647,7 +3154,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>SC_AS400_To_DropZone_MD</t>
+          <t>J_EyeMed_CMS_837_DBLoad_ODS</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -3665,12 +3172,12 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>SC_AS400_To_DropZone_MD</t>
+          <t>J_EyeMed_CMS_837_DBLoad_ODS</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>{'component': 'tJava', 'risk': 'HIGH', 'modernization': 'Rewrite using Talend native components', 'replacement': 'tMap / Talend Routine'}</t>
+          <t>{'component': 'tJavaRow', 'risk': 'HIGH', 'modernization': 'Replace with tMap expressions', 'replacement': 'tMap'}</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -3683,7 +3190,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>SC_AS400_To_DropZone_MD</t>
+          <t>J_EyeMed_CMS_837_DBLoad_ODS</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -3701,12 +3208,12 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>SC_AS400_To_DropZone_MD</t>
+          <t>J_EyeMed_CMS_837_DBLoad_ODS</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>{'component': 'tJava', 'risk': 'HIGH', 'modernization': 'Rewrite using Talend native components', 'replacement': 'tMap / Talend Routine'}</t>
+          <t>{'component': 'tJavaRow', 'risk': 'HIGH', 'modernization': 'Replace with tMap expressions', 'replacement': 'tMap'}</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -3719,12 +3226,12 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>SC_AS400_To_DropZone_MD</t>
+          <t>J_EyeMed_CMS_837_DBLoad_ODS</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>{'component': 'tJava', 'risk': 'HIGH', 'modernization': 'Rewrite using Talend native components', 'replacement': 'tMap / Talend Routine'}</t>
+          <t>{'component': 'tFTPGet', 'risk': 'MEDIUM', 'modernization': 'Replace with secure file transfer', 'replacement': 'tFTPFileList'}</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -3737,7 +3244,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>SC_AS400_To_DropZone_MD</t>
+          <t>J_EyeMed_CMS_837_DBLoad_ODS</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -3755,12 +3262,12 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>SC_AS400_To_DropZone_MD</t>
+          <t>J_EyeMed_CMS_837_DBLoad_ODS</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>{'component': 'tJavaRow', 'risk': 'HIGH', 'modernization': 'Replace with tMap expressions', 'replacement': 'tMap'}</t>
+          <t>{'component': 'tJava', 'risk': 'HIGH', 'modernization': 'Rewrite using Talend native components', 'replacement': 'tMap / Talend Routine'}</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -3773,7 +3280,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>SC_AS400_To_DropZone_MD</t>
+          <t>J_EyeMed_CMS_837_DBLoad_ODS</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -3791,7 +3298,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>SC_AS400_To_DropZone_MD</t>
+          <t>J_EyeMed_CMS_837_DBLoad_ODS</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -3809,7 +3316,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>SC_AS400_To_DropZone_MD</t>
+          <t>J_EyeMed_CMS_837_DBLoad_ODS</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -3827,7 +3334,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>SC_AS400_To_DropZone_MD</t>
+          <t>J_EyeMed_CMS_837_DBLoad_ODS</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -3845,12 +3352,12 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>SC_AS400_To_DropZone_MD</t>
+          <t>J_EyeMed_CMS_837_DBLoad_ODS</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>{'component': 'tJava', 'risk': 'HIGH', 'modernization': 'Rewrite using Talend native components', 'replacement': 'tMap / Talend Routine'}</t>
+          <t>{'component': 'tJavaRow', 'risk': 'HIGH', 'modernization': 'Replace with tMap expressions', 'replacement': 'tMap'}</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -3863,12 +3370,12 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>SC_AS400_To_DropZone_MD</t>
+          <t>J_EyeMed_CMS_837_DBLoad_ODS</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>{'component': 'tJava', 'risk': 'HIGH', 'modernization': 'Rewrite using Talend native components', 'replacement': 'tMap / Talend Routine'}</t>
+          <t>{'component': 'tFTPGet', 'risk': 'MEDIUM', 'modernization': 'Replace with secure file transfer', 'replacement': 'tFTPFileList'}</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -3881,12 +3388,12 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>SC_AS400_To_DropZone_MD</t>
+          <t>J_EyeMed_CMS_837_DBLoad_ODS</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>{'component': 'tJava', 'risk': 'HIGH', 'modernization': 'Rewrite using Talend native components', 'replacement': 'tMap / Talend Routine'}</t>
+          <t>{'component': 'tJavaRow', 'risk': 'HIGH', 'modernization': 'Replace with tMap expressions', 'replacement': 'tMap'}</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -3899,7 +3406,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>SC_AS400_To_DropZone_MD</t>
+          <t>J_EyeMed_CMS_837_DBLoad_ODS</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -3917,7 +3424,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>SC_AS400_To_DropZone_MD</t>
+          <t>J_EyeMed_CMS_837_DBLoad_ODS</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -3931,330 +3438,6 @@
         </is>
       </c>
       <c r="D17" t="inlineStr"/>
-    </row>
-    <row r="18">
-      <c r="A18" t="inlineStr">
-        <is>
-          <t>SC_AS400_To_DropZone_MD</t>
-        </is>
-      </c>
-      <c r="B18" t="inlineStr">
-        <is>
-          <t>{'component': 'tJavaRow', 'risk': 'HIGH', 'modernization': 'Replace with tMap expressions', 'replacement': 'tMap'}</t>
-        </is>
-      </c>
-      <c r="C18" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="D18" t="inlineStr"/>
-    </row>
-    <row r="19">
-      <c r="A19" t="inlineStr">
-        <is>
-          <t>SC_AS400_To_DropZone_MD</t>
-        </is>
-      </c>
-      <c r="B19" t="inlineStr">
-        <is>
-          <t>{'component': 'tJavaRow', 'risk': 'HIGH', 'modernization': 'Replace with tMap expressions', 'replacement': 'tMap'}</t>
-        </is>
-      </c>
-      <c r="C19" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="D19" t="inlineStr"/>
-    </row>
-    <row r="20">
-      <c r="A20" t="inlineStr">
-        <is>
-          <t>SC_AS400_To_DropZone_MD</t>
-        </is>
-      </c>
-      <c r="B20" t="inlineStr">
-        <is>
-          <t>{'component': 'tJava', 'risk': 'HIGH', 'modernization': 'Rewrite using Talend native components', 'replacement': 'tMap / Talend Routine'}</t>
-        </is>
-      </c>
-      <c r="C20" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="D20" t="inlineStr"/>
-    </row>
-    <row r="21">
-      <c r="A21" t="inlineStr">
-        <is>
-          <t>SC_AS400_To_DropZone_MD</t>
-        </is>
-      </c>
-      <c r="B21" t="inlineStr">
-        <is>
-          <t>{'component': 'tJava', 'risk': 'HIGH', 'modernization': 'Rewrite using Talend native components', 'replacement': 'tMap / Talend Routine'}</t>
-        </is>
-      </c>
-      <c r="C21" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="D21" t="inlineStr"/>
-    </row>
-    <row r="22">
-      <c r="A22" t="inlineStr">
-        <is>
-          <t>SC_AS400_To_DropZone_MD</t>
-        </is>
-      </c>
-      <c r="B22" t="inlineStr">
-        <is>
-          <t>{'component': 'tJavaRow', 'risk': 'HIGH', 'modernization': 'Replace with tMap expressions', 'replacement': 'tMap'}</t>
-        </is>
-      </c>
-      <c r="C22" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="D22" t="inlineStr"/>
-    </row>
-    <row r="23">
-      <c r="A23" t="inlineStr">
-        <is>
-          <t>SC_AS400_To_DropZone_MD</t>
-        </is>
-      </c>
-      <c r="B23" t="inlineStr">
-        <is>
-          <t>{'component': 'tJava', 'risk': 'HIGH', 'modernization': 'Rewrite using Talend native components', 'replacement': 'tMap / Talend Routine'}</t>
-        </is>
-      </c>
-      <c r="C23" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="D23" t="inlineStr"/>
-    </row>
-    <row r="24">
-      <c r="A24" t="inlineStr">
-        <is>
-          <t>SC_AS400_To_DropZone_MD</t>
-        </is>
-      </c>
-      <c r="B24" t="inlineStr">
-        <is>
-          <t>{'component': 'tJava', 'risk': 'HIGH', 'modernization': 'Rewrite using Talend native components', 'replacement': 'tMap / Talend Routine'}</t>
-        </is>
-      </c>
-      <c r="C24" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="D24" t="inlineStr"/>
-    </row>
-    <row r="25">
-      <c r="A25" t="inlineStr">
-        <is>
-          <t>SC_AS400_To_DropZone_MD</t>
-        </is>
-      </c>
-      <c r="B25" t="inlineStr">
-        <is>
-          <t>{'component': 'tJava', 'risk': 'HIGH', 'modernization': 'Rewrite using Talend native components', 'replacement': 'tMap / Talend Routine'}</t>
-        </is>
-      </c>
-      <c r="C25" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="D25" t="inlineStr"/>
-    </row>
-    <row r="26">
-      <c r="A26" t="inlineStr">
-        <is>
-          <t>SC_AS400_To_DropZone_MD</t>
-        </is>
-      </c>
-      <c r="B26" t="inlineStr">
-        <is>
-          <t>{'component': 'tJava', 'risk': 'HIGH', 'modernization': 'Rewrite using Talend native components', 'replacement': 'tMap / Talend Routine'}</t>
-        </is>
-      </c>
-      <c r="C26" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="D26" t="inlineStr"/>
-    </row>
-    <row r="27">
-      <c r="A27" t="inlineStr">
-        <is>
-          <t>SC_AS400_To_DropZone_MD</t>
-        </is>
-      </c>
-      <c r="B27" t="inlineStr">
-        <is>
-          <t>{'component': 'tJava', 'risk': 'HIGH', 'modernization': 'Rewrite using Talend native components', 'replacement': 'tMap / Talend Routine'}</t>
-        </is>
-      </c>
-      <c r="C27" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="D27" t="inlineStr"/>
-    </row>
-    <row r="28">
-      <c r="A28" t="inlineStr">
-        <is>
-          <t>SC_AS400_To_DropZone_MD</t>
-        </is>
-      </c>
-      <c r="B28" t="inlineStr">
-        <is>
-          <t>{'component': 'tJava', 'risk': 'HIGH', 'modernization': 'Rewrite using Talend native components', 'replacement': 'tMap / Talend Routine'}</t>
-        </is>
-      </c>
-      <c r="C28" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="D28" t="inlineStr"/>
-    </row>
-    <row r="29">
-      <c r="A29" t="inlineStr">
-        <is>
-          <t>SC_AS400_To_DropZone_MD</t>
-        </is>
-      </c>
-      <c r="B29" t="inlineStr">
-        <is>
-          <t>{'component': 'tJavaRow', 'risk': 'HIGH', 'modernization': 'Replace with tMap expressions', 'replacement': 'tMap'}</t>
-        </is>
-      </c>
-      <c r="C29" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="D29" t="inlineStr"/>
-    </row>
-    <row r="30">
-      <c r="A30" t="inlineStr">
-        <is>
-          <t>SC_AS400_To_DropZone_MD</t>
-        </is>
-      </c>
-      <c r="B30" t="inlineStr">
-        <is>
-          <t>{'component': 'tJavaRow', 'risk': 'HIGH', 'modernization': 'Replace with tMap expressions', 'replacement': 'tMap'}</t>
-        </is>
-      </c>
-      <c r="C30" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="D30" t="inlineStr"/>
-    </row>
-    <row r="31">
-      <c r="A31" t="inlineStr">
-        <is>
-          <t>SC_AS400_To_DropZone_MD</t>
-        </is>
-      </c>
-      <c r="B31" t="inlineStr">
-        <is>
-          <t>{'component': 'tJava', 'risk': 'HIGH', 'modernization': 'Rewrite using Talend native components', 'replacement': 'tMap / Talend Routine'}</t>
-        </is>
-      </c>
-      <c r="C31" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="D31" t="inlineStr"/>
-    </row>
-    <row r="32">
-      <c r="A32" t="inlineStr">
-        <is>
-          <t>SC_AS400_To_DropZone_MD</t>
-        </is>
-      </c>
-      <c r="B32" t="inlineStr">
-        <is>
-          <t>{'component': 'tJava', 'risk': 'HIGH', 'modernization': 'Rewrite using Talend native components', 'replacement': 'tMap / Talend Routine'}</t>
-        </is>
-      </c>
-      <c r="C32" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="D32" t="inlineStr"/>
-    </row>
-    <row r="33">
-      <c r="A33" t="inlineStr">
-        <is>
-          <t>SC_AS400_To_DropZone_MD</t>
-        </is>
-      </c>
-      <c r="B33" t="inlineStr">
-        <is>
-          <t>{'component': 'tJavaRow', 'risk': 'HIGH', 'modernization': 'Replace with tMap expressions', 'replacement': 'tMap'}</t>
-        </is>
-      </c>
-      <c r="C33" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="D33" t="inlineStr"/>
-    </row>
-    <row r="34">
-      <c r="A34" t="inlineStr">
-        <is>
-          <t>SC_AS400_To_DropZone_MD</t>
-        </is>
-      </c>
-      <c r="B34" t="inlineStr">
-        <is>
-          <t>{'component': 'tJava', 'risk': 'HIGH', 'modernization': 'Rewrite using Talend native components', 'replacement': 'tMap / Talend Routine'}</t>
-        </is>
-      </c>
-      <c r="C34" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="D34" t="inlineStr"/>
-    </row>
-    <row r="35">
-      <c r="A35" t="inlineStr">
-        <is>
-          <t>SC_AS400_To_DropZone_MD</t>
-        </is>
-      </c>
-      <c r="B35" t="inlineStr">
-        <is>
-          <t>{'component': 'tJavaRow', 'risk': 'HIGH', 'modernization': 'Replace with tMap expressions', 'replacement': 'tMap'}</t>
-        </is>
-      </c>
-      <c r="C35" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="D35" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
feat: one-click upload on home page - skip double upload prompt
</commit_message>
<xml_diff>
--- a/output/migration_report.xlsx
+++ b/output/migration_report.xlsx
@@ -455,7 +455,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
     </row>
@@ -479,7 +479,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>6</t>
         </is>
       </c>
     </row>
@@ -506,10 +506,10 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H3"/>
+  <dimension ref="A1:H4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="29" customWidth="1" min="1" max="1"/>
+    <col width="52" customWidth="1" min="1" max="1"/>
     <col width="10" customWidth="1" min="2" max="2"/>
     <col width="12" customWidth="1" min="3" max="3"/>
     <col width="12" customWidth="1" min="4" max="4"/>
@@ -564,16 +564,16 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>J_EyeMed_CMS_837_DBLoad_ODS</t>
+          <t>SC_Landing_To_Staging_Full_Load_CDP_Consumption_MD</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>0.17</t>
+          <t>0.3</t>
         </is>
       </c>
       <c r="C2" t="n">
-        <v>76</v>
+        <v>41</v>
       </c>
       <c r="D2" t="inlineStr"/>
       <c r="E2" t="inlineStr">
@@ -596,16 +596,16 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>J_EyeMed_CMS_837_DBLoad_ODS</t>
+          <t>SC_Landing_To_Staging_Full_Load_CDP_Consumption_MD</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>0.18</t>
+          <t>0.4</t>
         </is>
       </c>
       <c r="C3" t="n">
-        <v>76</v>
+        <v>41</v>
       </c>
       <c r="D3" t="inlineStr"/>
       <c r="E3" t="inlineStr">
@@ -622,6 +622,38 @@
         </is>
       </c>
       <c r="H3" t="n">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>SC_Landing_To_Staging_Full_Load_CDP_Consumption_MD</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>1.1</t>
+        </is>
+      </c>
+      <c r="C4" t="n">
+        <v>70</v>
+      </c>
+      <c r="D4" t="inlineStr"/>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>GREEN</t>
+        </is>
+      </c>
+      <c r="F4" t="n">
+        <v>2</v>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H4" t="n">
         <v>16</v>
       </c>
     </row>
@@ -636,10 +668,10 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E15"/>
+  <dimension ref="A1:E18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="29" customWidth="1" min="1" max="1"/>
+    <col width="52" customWidth="1" min="1" max="1"/>
     <col width="10" customWidth="1" min="2" max="2"/>
     <col width="11" customWidth="1" min="3" max="3"/>
     <col width="10" customWidth="1" min="4" max="4"/>
@@ -676,7 +708,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>J_EyeMed_CMS_837_DBLoad_ODS</t>
+          <t>SC_Landing_To_Staging_Full_Load_CDP_Consumption_MD</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -695,17 +727,17 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>J_EyeMed_CMS_837_DBLoad_ODS</t>
+          <t>SC_Landing_To_Staging_Full_Load_CDP_Consumption_MD</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>LOW</t>
+          <t>HIGH</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>tMap</t>
+          <t>tJavaRow</t>
         </is>
       </c>
       <c r="D3" t="inlineStr"/>
@@ -714,26 +746,26 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>J_EyeMed_CMS_837_DBLoad_ODS</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
+          <t>SC_Landing_To_Staging_Full_Load_CDP_Consumption_MD</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr"/>
       <c r="C4" t="inlineStr">
         <is>
-          <t>tJavaRow</t>
+          <t>tJava</t>
         </is>
       </c>
       <c r="D4" t="inlineStr"/>
-      <c r="E4" t="inlineStr"/>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>{'risk': 'HIGH', 'issue': 'Custom Java Code', 'recommendation': 'Requires manual remediation'}</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>J_EyeMed_CMS_837_DBLoad_ODS</t>
+          <t>SC_Landing_To_Staging_Full_Load_CDP_Consumption_MD</t>
         </is>
       </c>
       <c r="B5" t="inlineStr"/>
@@ -752,7 +784,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>J_EyeMed_CMS_837_DBLoad_ODS</t>
+          <t>SC_Landing_To_Staging_Full_Load_CDP_Consumption_MD</t>
         </is>
       </c>
       <c r="B6" t="inlineStr"/>
@@ -771,140 +803,140 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>J_EyeMed_CMS_837_DBLoad_ODS</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr"/>
+          <t>SC_Landing_To_Staging_Full_Load_CDP_Consumption_MD</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
       <c r="C7" t="inlineStr">
         <is>
           <t>tJava</t>
         </is>
       </c>
       <c r="D7" t="inlineStr"/>
-      <c r="E7" t="inlineStr">
-        <is>
-          <t>{'risk': 'HIGH', 'issue': 'Custom Java Code', 'recommendation': 'Requires manual remediation'}</t>
-        </is>
-      </c>
+      <c r="E7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>J_EyeMed_CMS_837_DBLoad_ODS</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr"/>
+          <t>SC_Landing_To_Staging_Full_Load_CDP_Consumption_MD</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>tJava</t>
+          <t>tJavaRow</t>
         </is>
       </c>
       <c r="D8" t="inlineStr"/>
-      <c r="E8" t="inlineStr">
-        <is>
-          <t>{'risk': 'HIGH', 'issue': 'Custom Java Code', 'recommendation': 'Requires manual remediation'}</t>
-        </is>
-      </c>
+      <c r="E8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>J_EyeMed_CMS_837_DBLoad_ODS</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
+          <t>SC_Landing_To_Staging_Full_Load_CDP_Consumption_MD</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr"/>
       <c r="C9" t="inlineStr">
         <is>
           <t>tJava</t>
         </is>
       </c>
       <c r="D9" t="inlineStr"/>
-      <c r="E9" t="inlineStr"/>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>{'risk': 'HIGH', 'issue': 'Custom Java Code', 'recommendation': 'Requires manual remediation'}</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>J_EyeMed_CMS_837_DBLoad_ODS</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>LOW</t>
-        </is>
-      </c>
+          <t>SC_Landing_To_Staging_Full_Load_CDP_Consumption_MD</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr"/>
       <c r="C10" t="inlineStr">
         <is>
-          <t>tMap</t>
+          <t>tJava</t>
         </is>
       </c>
       <c r="D10" t="inlineStr"/>
-      <c r="E10" t="inlineStr"/>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>{'risk': 'HIGH', 'issue': 'Custom Java Code', 'recommendation': 'Requires manual remediation'}</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>J_EyeMed_CMS_837_DBLoad_ODS</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
+          <t>SC_Landing_To_Staging_Full_Load_CDP_Consumption_MD</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr"/>
       <c r="C11" t="inlineStr">
         <is>
-          <t>tJavaRow</t>
+          <t>tJava</t>
         </is>
       </c>
       <c r="D11" t="inlineStr"/>
-      <c r="E11" t="inlineStr"/>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>{'risk': 'HIGH', 'issue': 'Custom Java Code', 'recommendation': 'Requires manual remediation'}</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>J_EyeMed_CMS_837_DBLoad_ODS</t>
-        </is>
-      </c>
-      <c r="B12" t="inlineStr"/>
+          <t>SC_Landing_To_Staging_Full_Load_CDP_Consumption_MD</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
       <c r="C12" t="inlineStr">
         <is>
           <t>tJava</t>
         </is>
       </c>
       <c r="D12" t="inlineStr"/>
-      <c r="E12" t="inlineStr">
-        <is>
-          <t>{'risk': 'HIGH', 'issue': 'Custom Java Code', 'recommendation': 'Requires manual remediation'}</t>
-        </is>
-      </c>
+      <c r="E12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>J_EyeMed_CMS_837_DBLoad_ODS</t>
-        </is>
-      </c>
-      <c r="B13" t="inlineStr"/>
+          <t>SC_Landing_To_Staging_Full_Load_CDP_Consumption_MD</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>tJava</t>
+          <t>tJavaRow</t>
         </is>
       </c>
       <c r="D13" t="inlineStr"/>
-      <c r="E13" t="inlineStr">
-        <is>
-          <t>{'risk': 'HIGH', 'issue': 'Custom Java Code', 'recommendation': 'Requires manual remediation'}</t>
-        </is>
-      </c>
+      <c r="E13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>J_EyeMed_CMS_837_DBLoad_ODS</t>
+          <t>SC_Landing_To_Staging_Full_Load_CDP_Consumption_MD</t>
         </is>
       </c>
       <c r="B14" t="inlineStr"/>
@@ -923,7 +955,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>J_EyeMed_CMS_837_DBLoad_ODS</t>
+          <t>SC_Landing_To_Staging_Full_Load_CDP_Consumption_MD</t>
         </is>
       </c>
       <c r="B15" t="inlineStr"/>
@@ -934,6 +966,63 @@
       </c>
       <c r="D15" t="inlineStr"/>
       <c r="E15" t="inlineStr">
+        <is>
+          <t>{'risk': 'HIGH', 'issue': 'Custom Java Code', 'recommendation': 'Requires manual remediation'}</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>SC_Landing_To_Staging_Full_Load_CDP_Consumption_MD</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr"/>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>tJava</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr"/>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>{'risk': 'HIGH', 'issue': 'Custom Java Code', 'recommendation': 'Requires manual remediation'}</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>SC_Landing_To_Staging_Full_Load_CDP_Consumption_MD</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr"/>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>tJava</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr"/>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>{'risk': 'HIGH', 'issue': 'Custom Java Code', 'recommendation': 'Requires manual remediation'}</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>SC_Landing_To_Staging_Full_Load_CDP_Consumption_MD</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr"/>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>tJava</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr"/>
+      <c r="E18" t="inlineStr">
         <is>
           <t>{'risk': 'HIGH', 'issue': 'Custom Java Code', 'recommendation': 'Requires manual remediation'}</t>
         </is>
@@ -953,9 +1042,9 @@
   <dimension ref="A1:D153"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="29" customWidth="1" min="1" max="1"/>
+    <col width="52" customWidth="1" min="1" max="1"/>
     <col width="16" customWidth="1" min="2" max="2"/>
-    <col width="21" customWidth="1" min="3" max="3"/>
+    <col width="25" customWidth="1" min="3" max="3"/>
     <col width="10" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
@@ -984,13 +1073,13 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>J_EyeMed_CMS_837_DBLoad_ODS</t>
+          <t>SC_Landing_To_Staging_Full_Load_CDP_Consumption_MD</t>
         </is>
       </c>
       <c r="B2" t="inlineStr"/>
       <c r="C2" t="inlineStr">
         <is>
-          <t>tMSSqlConnection</t>
+          <t>tPrejob</t>
         </is>
       </c>
       <c r="D2" t="inlineStr"/>
@@ -998,13 +1087,13 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>J_EyeMed_CMS_837_DBLoad_ODS</t>
+          <t>SC_Landing_To_Staging_Full_Load_CDP_Consumption_MD</t>
         </is>
       </c>
       <c r="B3" t="inlineStr"/>
       <c r="C3" t="inlineStr">
         <is>
-          <t>tFileList</t>
+          <t>tJava</t>
         </is>
       </c>
       <c r="D3" t="inlineStr"/>
@@ -1012,13 +1101,13 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>J_EyeMed_CMS_837_DBLoad_ODS</t>
+          <t>SC_Landing_To_Staging_Full_Load_CDP_Consumption_MD</t>
         </is>
       </c>
       <c r="B4" t="inlineStr"/>
       <c r="C4" t="inlineStr">
         <is>
-          <t>tFileInputRaw</t>
+          <t>tMysqlConnection</t>
         </is>
       </c>
       <c r="D4" t="inlineStr"/>
@@ -1026,13 +1115,13 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>J_EyeMed_CMS_837_DBLoad_ODS</t>
+          <t>SC_Landing_To_Staging_Full_Load_CDP_Consumption_MD</t>
         </is>
       </c>
       <c r="B5" t="inlineStr"/>
       <c r="C5" t="inlineStr">
         <is>
-          <t>tHMap</t>
+          <t>tJava</t>
         </is>
       </c>
       <c r="D5" t="inlineStr"/>
@@ -1040,13 +1129,13 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>J_EyeMed_CMS_837_DBLoad_ODS</t>
+          <t>SC_Landing_To_Staging_Full_Load_CDP_Consumption_MD</t>
         </is>
       </c>
       <c r="B6" t="inlineStr"/>
       <c r="C6" t="inlineStr">
         <is>
-          <t>tFileOutputRaw</t>
+          <t>tMysqlInput</t>
         </is>
       </c>
       <c r="D6" t="inlineStr"/>
@@ -1054,13 +1143,13 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>J_EyeMed_CMS_837_DBLoad_ODS</t>
+          <t>SC_Landing_To_Staging_Full_Load_CDP_Consumption_MD</t>
         </is>
       </c>
       <c r="B7" t="inlineStr"/>
       <c r="C7" t="inlineStr">
         <is>
-          <t>tDie</t>
+          <t>tFlowToIterate</t>
         </is>
       </c>
       <c r="D7" t="inlineStr"/>
@@ -1068,13 +1157,13 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>J_EyeMed_CMS_837_DBLoad_ODS</t>
+          <t>SC_Landing_To_Staging_Full_Load_CDP_Consumption_MD</t>
         </is>
       </c>
       <c r="B8" t="inlineStr"/>
       <c r="C8" t="inlineStr">
         <is>
-          <t>tFileList</t>
+          <t>tJava</t>
         </is>
       </c>
       <c r="D8" t="inlineStr"/>
@@ -1082,13 +1171,13 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>J_EyeMed_CMS_837_DBLoad_ODS</t>
+          <t>SC_Landing_To_Staging_Full_Load_CDP_Consumption_MD</t>
         </is>
       </c>
       <c r="B9" t="inlineStr"/>
       <c r="C9" t="inlineStr">
         <is>
-          <t>tJava</t>
+          <t>tImpalaConnection</t>
         </is>
       </c>
       <c r="D9" t="inlineStr"/>
@@ -1096,13 +1185,13 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>J_EyeMed_CMS_837_DBLoad_ODS</t>
+          <t>SC_Landing_To_Staging_Full_Load_CDP_Consumption_MD</t>
         </is>
       </c>
       <c r="B10" t="inlineStr"/>
       <c r="C10" t="inlineStr">
         <is>
-          <t>tMSSqlInput</t>
+          <t>tImpalaRow</t>
         </is>
       </c>
       <c r="D10" t="inlineStr"/>
@@ -1110,13 +1199,13 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>J_EyeMed_CMS_837_DBLoad_ODS</t>
+          <t>SC_Landing_To_Staging_Full_Load_CDP_Consumption_MD</t>
         </is>
       </c>
       <c r="B11" t="inlineStr"/>
       <c r="C11" t="inlineStr">
         <is>
-          <t>tMap</t>
+          <t>tImpalaInput</t>
         </is>
       </c>
       <c r="D11" t="inlineStr"/>
@@ -1124,13 +1213,13 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>J_EyeMed_CMS_837_DBLoad_ODS</t>
+          <t>SC_Landing_To_Staging_Full_Load_CDP_Consumption_MD</t>
         </is>
       </c>
       <c r="B12" t="inlineStr"/>
       <c r="C12" t="inlineStr">
         <is>
-          <t>tSetGlobalVar</t>
+          <t>tJavaRow</t>
         </is>
       </c>
       <c r="D12" t="inlineStr"/>
@@ -1138,13 +1227,13 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>J_EyeMed_CMS_837_DBLoad_ODS</t>
+          <t>SC_Landing_To_Staging_Full_Load_CDP_Consumption_MD</t>
         </is>
       </c>
       <c r="B13" t="inlineStr"/>
       <c r="C13" t="inlineStr">
         <is>
-          <t>tFileInputXML</t>
+          <t>Job_Start</t>
         </is>
       </c>
       <c r="D13" t="inlineStr"/>
@@ -1152,13 +1241,13 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>J_EyeMed_CMS_837_DBLoad_ODS</t>
+          <t>SC_Landing_To_Staging_Full_Load_CDP_Consumption_MD</t>
         </is>
       </c>
       <c r="B14" t="inlineStr"/>
       <c r="C14" t="inlineStr">
         <is>
-          <t>tMap</t>
+          <t>Implicit_context_joblet</t>
         </is>
       </c>
       <c r="D14" t="inlineStr"/>
@@ -1166,13 +1255,13 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>J_EyeMed_CMS_837_DBLoad_ODS</t>
+          <t>SC_Landing_To_Staging_Full_Load_CDP_Consumption_MD</t>
         </is>
       </c>
       <c r="B15" t="inlineStr"/>
       <c r="C15" t="inlineStr">
         <is>
-          <t>tMap</t>
+          <t>tDie</t>
         </is>
       </c>
       <c r="D15" t="inlineStr"/>
@@ -1180,13 +1269,13 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>J_EyeMed_CMS_837_DBLoad_ODS</t>
+          <t>SC_Landing_To_Staging_Full_Load_CDP_Consumption_MD</t>
         </is>
       </c>
       <c r="B16" t="inlineStr"/>
       <c r="C16" t="inlineStr">
         <is>
-          <t>tHashInput</t>
+          <t>tDie</t>
         </is>
       </c>
       <c r="D16" t="inlineStr"/>
@@ -1194,13 +1283,13 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>J_EyeMed_CMS_837_DBLoad_ODS</t>
+          <t>SC_Landing_To_Staging_Full_Load_CDP_Consumption_MD</t>
         </is>
       </c>
       <c r="B17" t="inlineStr"/>
       <c r="C17" t="inlineStr">
         <is>
-          <t>tMSSqlOutput</t>
+          <t>tMysqlInput</t>
         </is>
       </c>
       <c r="D17" t="inlineStr"/>
@@ -1208,13 +1297,13 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>J_EyeMed_CMS_837_DBLoad_ODS</t>
+          <t>SC_Landing_To_Staging_Full_Load_CDP_Consumption_MD</t>
         </is>
       </c>
       <c r="B18" t="inlineStr"/>
       <c r="C18" t="inlineStr">
         <is>
-          <t>tFileInputXML</t>
+          <t>tJavaRow</t>
         </is>
       </c>
       <c r="D18" t="inlineStr"/>
@@ -1222,13 +1311,13 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>J_EyeMed_CMS_837_DBLoad_ODS</t>
+          <t>SC_Landing_To_Staging_Full_Load_CDP_Consumption_MD</t>
         </is>
       </c>
       <c r="B19" t="inlineStr"/>
       <c r="C19" t="inlineStr">
         <is>
-          <t>tMap</t>
+          <t>tFixedFlowInput</t>
         </is>
       </c>
       <c r="D19" t="inlineStr"/>
@@ -1236,13 +1325,13 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>J_EyeMed_CMS_837_DBLoad_ODS</t>
+          <t>SC_Landing_To_Staging_Full_Load_CDP_Consumption_MD</t>
         </is>
       </c>
       <c r="B20" t="inlineStr"/>
       <c r="C20" t="inlineStr">
         <is>
-          <t>tMap</t>
+          <t>tLogRow</t>
         </is>
       </c>
       <c r="D20" t="inlineStr"/>
@@ -1250,13 +1339,13 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>J_EyeMed_CMS_837_DBLoad_ODS</t>
+          <t>SC_Landing_To_Staging_Full_Load_CDP_Consumption_MD</t>
         </is>
       </c>
       <c r="B21" t="inlineStr"/>
       <c r="C21" t="inlineStr">
         <is>
-          <t>tHashInput</t>
+          <t>tMysqlOutput</t>
         </is>
       </c>
       <c r="D21" t="inlineStr"/>
@@ -1264,13 +1353,13 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>J_EyeMed_CMS_837_DBLoad_ODS</t>
+          <t>SC_Landing_To_Staging_Full_Load_CDP_Consumption_MD</t>
         </is>
       </c>
       <c r="B22" t="inlineStr"/>
       <c r="C22" t="inlineStr">
         <is>
-          <t>tMSSqlOutput</t>
+          <t>Job_End</t>
         </is>
       </c>
       <c r="D22" t="inlineStr"/>
@@ -1278,13 +1367,13 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>J_EyeMed_CMS_837_DBLoad_ODS</t>
+          <t>SC_Landing_To_Staging_Full_Load_CDP_Consumption_MD</t>
         </is>
       </c>
       <c r="B23" t="inlineStr"/>
       <c r="C23" t="inlineStr">
         <is>
-          <t>tFileInputXML</t>
+          <t>tMysqlInput</t>
         </is>
       </c>
       <c r="D23" t="inlineStr"/>
@@ -1292,13 +1381,13 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>J_EyeMed_CMS_837_DBLoad_ODS</t>
+          <t>SC_Landing_To_Staging_Full_Load_CDP_Consumption_MD</t>
         </is>
       </c>
       <c r="B24" t="inlineStr"/>
       <c r="C24" t="inlineStr">
         <is>
-          <t>tMap</t>
+          <t>tFlowToIterate</t>
         </is>
       </c>
       <c r="D24" t="inlineStr"/>
@@ -1306,13 +1395,13 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>J_EyeMed_CMS_837_DBLoad_ODS</t>
+          <t>SC_Landing_To_Staging_Full_Load_CDP_Consumption_MD</t>
         </is>
       </c>
       <c r="B25" t="inlineStr"/>
       <c r="C25" t="inlineStr">
         <is>
-          <t>tMap</t>
+          <t>tMysqlInput</t>
         </is>
       </c>
       <c r="D25" t="inlineStr"/>
@@ -1320,13 +1409,13 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>J_EyeMed_CMS_837_DBLoad_ODS</t>
+          <t>SC_Landing_To_Staging_Full_Load_CDP_Consumption_MD</t>
         </is>
       </c>
       <c r="B26" t="inlineStr"/>
       <c r="C26" t="inlineStr">
         <is>
-          <t>tHashInput</t>
+          <t>tJavaRow</t>
         </is>
       </c>
       <c r="D26" t="inlineStr"/>
@@ -1334,13 +1423,13 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>J_EyeMed_CMS_837_DBLoad_ODS</t>
+          <t>SC_Landing_To_Staging_Full_Load_CDP_Consumption_MD</t>
         </is>
       </c>
       <c r="B27" t="inlineStr"/>
       <c r="C27" t="inlineStr">
         <is>
-          <t>tMSSqlOutput</t>
+          <t>tSendMail</t>
         </is>
       </c>
       <c r="D27" t="inlineStr"/>
@@ -1348,13 +1437,13 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>J_EyeMed_CMS_837_DBLoad_ODS</t>
+          <t>SC_Landing_To_Staging_Full_Load_CDP_Consumption_MD</t>
         </is>
       </c>
       <c r="B28" t="inlineStr"/>
       <c r="C28" t="inlineStr">
         <is>
-          <t>tFixedFlowInput</t>
+          <t>tImpalaRow</t>
         </is>
       </c>
       <c r="D28" t="inlineStr"/>
@@ -1362,13 +1451,13 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>J_EyeMed_CMS_837_DBLoad_ODS</t>
+          <t>SC_Landing_To_Staging_Full_Load_CDP_Consumption_MD</t>
         </is>
       </c>
       <c r="B29" t="inlineStr"/>
       <c r="C29" t="inlineStr">
         <is>
-          <t>tJavaRow</t>
+          <t>tPostjob</t>
         </is>
       </c>
       <c r="D29" t="inlineStr"/>
@@ -1376,13 +1465,13 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>J_EyeMed_CMS_837_DBLoad_ODS</t>
+          <t>SC_Landing_To_Staging_Full_Load_CDP_Consumption_MD</t>
         </is>
       </c>
       <c r="B30" t="inlineStr"/>
       <c r="C30" t="inlineStr">
         <is>
-          <t>tFileList</t>
+          <t>tImpalaClose</t>
         </is>
       </c>
       <c r="D30" t="inlineStr"/>
@@ -1390,13 +1479,13 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>J_EyeMed_CMS_837_DBLoad_ODS</t>
+          <t>SC_Landing_To_Staging_Full_Load_CDP_Consumption_MD</t>
         </is>
       </c>
       <c r="B31" t="inlineStr"/>
       <c r="C31" t="inlineStr">
         <is>
-          <t>tFileCopy</t>
+          <t>tMysqlClose</t>
         </is>
       </c>
       <c r="D31" t="inlineStr"/>
@@ -1404,13 +1493,13 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>J_EyeMed_CMS_837_DBLoad_ODS</t>
+          <t>SC_Landing_To_Staging_Full_Load_CDP_Consumption_MD</t>
         </is>
       </c>
       <c r="B32" t="inlineStr"/>
       <c r="C32" t="inlineStr">
         <is>
-          <t>tJava</t>
+          <t>Job_Error</t>
         </is>
       </c>
       <c r="D32" t="inlineStr"/>
@@ -1418,13 +1507,13 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>J_EyeMed_CMS_837_DBLoad_ODS</t>
+          <t>SC_Landing_To_Staging_Full_Load_CDP_Consumption_MD</t>
         </is>
       </c>
       <c r="B33" t="inlineStr"/>
       <c r="C33" t="inlineStr">
         <is>
-          <t>tSendMail</t>
+          <t>tFixedFlowInput</t>
         </is>
       </c>
       <c r="D33" t="inlineStr"/>
@@ -1432,13 +1521,13 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>J_EyeMed_CMS_837_DBLoad_ODS</t>
+          <t>SC_Landing_To_Staging_Full_Load_CDP_Consumption_MD</t>
         </is>
       </c>
       <c r="B34" t="inlineStr"/>
       <c r="C34" t="inlineStr">
         <is>
-          <t>tFileInputXML</t>
+          <t>tFlowToIterate</t>
         </is>
       </c>
       <c r="D34" t="inlineStr"/>
@@ -1446,13 +1535,13 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>J_EyeMed_CMS_837_DBLoad_ODS</t>
+          <t>SC_Landing_To_Staging_Full_Load_CDP_Consumption_MD</t>
         </is>
       </c>
       <c r="B35" t="inlineStr"/>
       <c r="C35" t="inlineStr">
         <is>
-          <t>tMap</t>
+          <t>tImpalaInput</t>
         </is>
       </c>
       <c r="D35" t="inlineStr"/>
@@ -1460,13 +1549,13 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>J_EyeMed_CMS_837_DBLoad_ODS</t>
+          <t>SC_Landing_To_Staging_Full_Load_CDP_Consumption_MD</t>
         </is>
       </c>
       <c r="B36" t="inlineStr"/>
       <c r="C36" t="inlineStr">
         <is>
-          <t>tMap</t>
+          <t>tJavaRow</t>
         </is>
       </c>
       <c r="D36" t="inlineStr"/>
@@ -1474,13 +1563,13 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>J_EyeMed_CMS_837_DBLoad_ODS</t>
+          <t>SC_Landing_To_Staging_Full_Load_CDP_Consumption_MD</t>
         </is>
       </c>
       <c r="B37" t="inlineStr"/>
       <c r="C37" t="inlineStr">
         <is>
-          <t>tMSSqlOutput</t>
+          <t>tImpalaRow</t>
         </is>
       </c>
       <c r="D37" t="inlineStr"/>
@@ -1488,13 +1577,13 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>J_EyeMed_CMS_837_DBLoad_ODS</t>
+          <t>SC_Landing_To_Staging_Full_Load_CDP_Consumption_MD</t>
         </is>
       </c>
       <c r="B38" t="inlineStr"/>
       <c r="C38" t="inlineStr">
         <is>
-          <t>tFileInputDelimited</t>
+          <t>tImpalaRow</t>
         </is>
       </c>
       <c r="D38" t="inlineStr"/>
@@ -1502,13 +1591,13 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>J_EyeMed_CMS_837_DBLoad_ODS</t>
+          <t>SC_Landing_To_Staging_Full_Load_CDP_Consumption_MD</t>
         </is>
       </c>
       <c r="B39" t="inlineStr"/>
       <c r="C39" t="inlineStr">
         <is>
-          <t>tJavaRow</t>
+          <t>tMysqlInput</t>
         </is>
       </c>
       <c r="D39" t="inlineStr"/>
@@ -1516,13 +1605,13 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>J_EyeMed_CMS_837_DBLoad_ODS</t>
+          <t>SC_Landing_To_Staging_Full_Load_CDP_Consumption_MD</t>
         </is>
       </c>
       <c r="B40" t="inlineStr"/>
       <c r="C40" t="inlineStr">
         <is>
-          <t>tFileInputXML</t>
+          <t>tMysqlInput</t>
         </is>
       </c>
       <c r="D40" t="inlineStr"/>
@@ -1530,13 +1619,13 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>J_EyeMed_CMS_837_DBLoad_ODS</t>
+          <t>SC_Landing_To_Staging_Full_Load_CDP_Consumption_MD</t>
         </is>
       </c>
       <c r="B41" t="inlineStr"/>
       <c r="C41" t="inlineStr">
         <is>
-          <t>tMap</t>
+          <t>tImpalaRow</t>
         </is>
       </c>
       <c r="D41" t="inlineStr"/>
@@ -1544,13 +1633,13 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>J_EyeMed_CMS_837_DBLoad_ODS</t>
+          <t>SC_Landing_To_Staging_Full_Load_CDP_Consumption_MD</t>
         </is>
       </c>
       <c r="B42" t="inlineStr"/>
       <c r="C42" t="inlineStr">
         <is>
-          <t>tMap</t>
+          <t>tImpalaRow</t>
         </is>
       </c>
       <c r="D42" t="inlineStr"/>
@@ -1558,13 +1647,13 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>J_EyeMed_CMS_837_DBLoad_ODS</t>
+          <t>SC_Landing_To_Staging_Full_Load_CDP_Consumption_MD</t>
         </is>
       </c>
       <c r="B43" t="inlineStr"/>
       <c r="C43" t="inlineStr">
         <is>
-          <t>tMSSqlInput</t>
+          <t>tPrejob</t>
         </is>
       </c>
       <c r="D43" t="inlineStr"/>
@@ -1572,13 +1661,13 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>J_EyeMed_CMS_837_DBLoad_ODS</t>
+          <t>SC_Landing_To_Staging_Full_Load_CDP_Consumption_MD</t>
         </is>
       </c>
       <c r="B44" t="inlineStr"/>
       <c r="C44" t="inlineStr">
         <is>
-          <t>tMSSqlOutput</t>
+          <t>tJava</t>
         </is>
       </c>
       <c r="D44" t="inlineStr"/>
@@ -1586,13 +1675,13 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>J_EyeMed_CMS_837_DBLoad_ODS</t>
+          <t>SC_Landing_To_Staging_Full_Load_CDP_Consumption_MD</t>
         </is>
       </c>
       <c r="B45" t="inlineStr"/>
       <c r="C45" t="inlineStr">
         <is>
-          <t>tFTPConnection</t>
+          <t>tMysqlConnection</t>
         </is>
       </c>
       <c r="D45" t="inlineStr"/>
@@ -1600,13 +1689,13 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>J_EyeMed_CMS_837_DBLoad_ODS</t>
+          <t>SC_Landing_To_Staging_Full_Load_CDP_Consumption_MD</t>
         </is>
       </c>
       <c r="B46" t="inlineStr"/>
       <c r="C46" t="inlineStr">
         <is>
-          <t>tFTPFileList</t>
+          <t>tJava</t>
         </is>
       </c>
       <c r="D46" t="inlineStr"/>
@@ -1614,13 +1703,13 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>J_EyeMed_CMS_837_DBLoad_ODS</t>
+          <t>SC_Landing_To_Staging_Full_Load_CDP_Consumption_MD</t>
         </is>
       </c>
       <c r="B47" t="inlineStr"/>
       <c r="C47" t="inlineStr">
         <is>
-          <t>tFTPGet</t>
+          <t>tMysqlInput</t>
         </is>
       </c>
       <c r="D47" t="inlineStr"/>
@@ -1628,13 +1717,13 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>J_EyeMed_CMS_837_DBLoad_ODS</t>
+          <t>SC_Landing_To_Staging_Full_Load_CDP_Consumption_MD</t>
         </is>
       </c>
       <c r="B48" t="inlineStr"/>
       <c r="C48" t="inlineStr">
         <is>
-          <t>tSendMail</t>
+          <t>tFlowToIterate</t>
         </is>
       </c>
       <c r="D48" t="inlineStr"/>
@@ -1642,13 +1731,13 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>J_EyeMed_CMS_837_DBLoad_ODS</t>
+          <t>SC_Landing_To_Staging_Full_Load_CDP_Consumption_MD</t>
         </is>
       </c>
       <c r="B49" t="inlineStr"/>
       <c r="C49" t="inlineStr">
         <is>
-          <t>tSendMail</t>
+          <t>tJava</t>
         </is>
       </c>
       <c r="D49" t="inlineStr"/>
@@ -1656,13 +1745,13 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>J_EyeMed_CMS_837_DBLoad_ODS</t>
+          <t>SC_Landing_To_Staging_Full_Load_CDP_Consumption_MD</t>
         </is>
       </c>
       <c r="B50" t="inlineStr"/>
       <c r="C50" t="inlineStr">
         <is>
-          <t>tDie</t>
+          <t>tImpalaConnection</t>
         </is>
       </c>
       <c r="D50" t="inlineStr"/>
@@ -1670,13 +1759,13 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>J_EyeMed_CMS_837_DBLoad_ODS</t>
+          <t>SC_Landing_To_Staging_Full_Load_CDP_Consumption_MD</t>
         </is>
       </c>
       <c r="B51" t="inlineStr"/>
       <c r="C51" t="inlineStr">
         <is>
-          <t>tPrejob</t>
+          <t>tImpalaRow</t>
         </is>
       </c>
       <c r="D51" t="inlineStr"/>
@@ -1684,13 +1773,13 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>J_EyeMed_CMS_837_DBLoad_ODS</t>
+          <t>SC_Landing_To_Staging_Full_Load_CDP_Consumption_MD</t>
         </is>
       </c>
       <c r="B52" t="inlineStr"/>
       <c r="C52" t="inlineStr">
         <is>
-          <t>tMSSqlConnection</t>
+          <t>tImpalaInput</t>
         </is>
       </c>
       <c r="D52" t="inlineStr"/>
@@ -1698,13 +1787,13 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>J_EyeMed_CMS_837_DBLoad_ODS</t>
+          <t>SC_Landing_To_Staging_Full_Load_CDP_Consumption_MD</t>
         </is>
       </c>
       <c r="B53" t="inlineStr"/>
       <c r="C53" t="inlineStr">
         <is>
-          <t>tStatCatcher</t>
+          <t>tJavaRow</t>
         </is>
       </c>
       <c r="D53" t="inlineStr"/>
@@ -1712,13 +1801,13 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>J_EyeMed_CMS_837_DBLoad_ODS</t>
+          <t>SC_Landing_To_Staging_Full_Load_CDP_Consumption_MD</t>
         </is>
       </c>
       <c r="B54" t="inlineStr"/>
       <c r="C54" t="inlineStr">
         <is>
-          <t>tMap</t>
+          <t>Job_Start</t>
         </is>
       </c>
       <c r="D54" t="inlineStr"/>
@@ -1726,13 +1815,13 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>J_EyeMed_CMS_837_DBLoad_ODS</t>
+          <t>SC_Landing_To_Staging_Full_Load_CDP_Consumption_MD</t>
         </is>
       </c>
       <c r="B55" t="inlineStr"/>
       <c r="C55" t="inlineStr">
         <is>
-          <t>tFlowToIterate</t>
+          <t>Implicit_context_joblet</t>
         </is>
       </c>
       <c r="D55" t="inlineStr"/>
@@ -1740,13 +1829,13 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>J_EyeMed_CMS_837_DBLoad_ODS</t>
+          <t>SC_Landing_To_Staging_Full_Load_CDP_Consumption_MD</t>
         </is>
       </c>
       <c r="B56" t="inlineStr"/>
       <c r="C56" t="inlineStr">
         <is>
-          <t>tJavaRow</t>
+          <t>tDie</t>
         </is>
       </c>
       <c r="D56" t="inlineStr"/>
@@ -1754,13 +1843,13 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>J_EyeMed_CMS_837_DBLoad_ODS</t>
+          <t>SC_Landing_To_Staging_Full_Load_CDP_Consumption_MD</t>
         </is>
       </c>
       <c r="B57" t="inlineStr"/>
       <c r="C57" t="inlineStr">
         <is>
-          <t>tMSSqlOutput</t>
+          <t>tDie</t>
         </is>
       </c>
       <c r="D57" t="inlineStr"/>
@@ -1768,13 +1857,13 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>J_EyeMed_CMS_837_DBLoad_ODS</t>
+          <t>SC_Landing_To_Staging_Full_Load_CDP_Consumption_MD</t>
         </is>
       </c>
       <c r="B58" t="inlineStr"/>
       <c r="C58" t="inlineStr">
         <is>
-          <t>tSendMail</t>
+          <t>tMysqlInput</t>
         </is>
       </c>
       <c r="D58" t="inlineStr"/>
@@ -1782,13 +1871,13 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>J_EyeMed_CMS_837_DBLoad_ODS</t>
+          <t>SC_Landing_To_Staging_Full_Load_CDP_Consumption_MD</t>
         </is>
       </c>
       <c r="B59" t="inlineStr"/>
       <c r="C59" t="inlineStr">
         <is>
-          <t>tLogCatcher</t>
+          <t>tJavaRow</t>
         </is>
       </c>
       <c r="D59" t="inlineStr"/>
@@ -1796,13 +1885,13 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>J_EyeMed_CMS_837_DBLoad_ODS</t>
+          <t>SC_Landing_To_Staging_Full_Load_CDP_Consumption_MD</t>
         </is>
       </c>
       <c r="B60" t="inlineStr"/>
       <c r="C60" t="inlineStr">
         <is>
-          <t>tMap</t>
+          <t>tFixedFlowInput</t>
         </is>
       </c>
       <c r="D60" t="inlineStr"/>
@@ -1810,13 +1899,13 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>J_EyeMed_CMS_837_DBLoad_ODS</t>
+          <t>SC_Landing_To_Staging_Full_Load_CDP_Consumption_MD</t>
         </is>
       </c>
       <c r="B61" t="inlineStr"/>
       <c r="C61" t="inlineStr">
         <is>
-          <t>tFlowToIterate</t>
+          <t>tLogRow</t>
         </is>
       </c>
       <c r="D61" t="inlineStr"/>
@@ -1824,13 +1913,13 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>J_EyeMed_CMS_837_DBLoad_ODS</t>
+          <t>SC_Landing_To_Staging_Full_Load_CDP_Consumption_MD</t>
         </is>
       </c>
       <c r="B62" t="inlineStr"/>
       <c r="C62" t="inlineStr">
         <is>
-          <t>tMSSqlOutput</t>
+          <t>tMysqlOutput</t>
         </is>
       </c>
       <c r="D62" t="inlineStr"/>
@@ -1838,13 +1927,13 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>J_EyeMed_CMS_837_DBLoad_ODS</t>
+          <t>SC_Landing_To_Staging_Full_Load_CDP_Consumption_MD</t>
         </is>
       </c>
       <c r="B63" t="inlineStr"/>
       <c r="C63" t="inlineStr">
         <is>
-          <t>tSendMail</t>
+          <t>Job_End</t>
         </is>
       </c>
       <c r="D63" t="inlineStr"/>
@@ -1852,13 +1941,13 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>J_EyeMed_CMS_837_DBLoad_ODS</t>
+          <t>SC_Landing_To_Staging_Full_Load_CDP_Consumption_MD</t>
         </is>
       </c>
       <c r="B64" t="inlineStr"/>
       <c r="C64" t="inlineStr">
         <is>
-          <t>tDie</t>
+          <t>tMysqlInput</t>
         </is>
       </c>
       <c r="D64" t="inlineStr"/>
@@ -1866,13 +1955,13 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>J_EyeMed_CMS_837_DBLoad_ODS</t>
+          <t>SC_Landing_To_Staging_Full_Load_CDP_Consumption_MD</t>
         </is>
       </c>
       <c r="B65" t="inlineStr"/>
       <c r="C65" t="inlineStr">
         <is>
-          <t>tFTPDelete</t>
+          <t>tFlowToIterate</t>
         </is>
       </c>
       <c r="D65" t="inlineStr"/>
@@ -1880,13 +1969,13 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>J_EyeMed_CMS_837_DBLoad_ODS</t>
+          <t>SC_Landing_To_Staging_Full_Load_CDP_Consumption_MD</t>
         </is>
       </c>
       <c r="B66" t="inlineStr"/>
       <c r="C66" t="inlineStr">
         <is>
-          <t>tFileInputXML</t>
+          <t>tMysqlInput</t>
         </is>
       </c>
       <c r="D66" t="inlineStr"/>
@@ -1894,13 +1983,13 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>J_EyeMed_CMS_837_DBLoad_ODS</t>
+          <t>SC_Landing_To_Staging_Full_Load_CDP_Consumption_MD</t>
         </is>
       </c>
       <c r="B67" t="inlineStr"/>
       <c r="C67" t="inlineStr">
         <is>
-          <t>tMap</t>
+          <t>tJavaRow</t>
         </is>
       </c>
       <c r="D67" t="inlineStr"/>
@@ -1908,13 +1997,13 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>J_EyeMed_CMS_837_DBLoad_ODS</t>
+          <t>SC_Landing_To_Staging_Full_Load_CDP_Consumption_MD</t>
         </is>
       </c>
       <c r="B68" t="inlineStr"/>
       <c r="C68" t="inlineStr">
         <is>
-          <t>tHashOutput</t>
+          <t>tSendMail</t>
         </is>
       </c>
       <c r="D68" t="inlineStr"/>
@@ -1922,13 +2011,13 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>J_EyeMed_CMS_837_DBLoad_ODS</t>
+          <t>SC_Landing_To_Staging_Full_Load_CDP_Consumption_MD</t>
         </is>
       </c>
       <c r="B69" t="inlineStr"/>
       <c r="C69" t="inlineStr">
         <is>
-          <t>tPostjob</t>
+          <t>tImpalaRow</t>
         </is>
       </c>
       <c r="D69" t="inlineStr"/>
@@ -1936,13 +2025,13 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>J_EyeMed_CMS_837_DBLoad_ODS</t>
+          <t>SC_Landing_To_Staging_Full_Load_CDP_Consumption_MD</t>
         </is>
       </c>
       <c r="B70" t="inlineStr"/>
       <c r="C70" t="inlineStr">
         <is>
-          <t>tMSSqlClose</t>
+          <t>tPostjob</t>
         </is>
       </c>
       <c r="D70" t="inlineStr"/>
@@ -1950,13 +2039,13 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>J_EyeMed_CMS_837_DBLoad_ODS</t>
+          <t>SC_Landing_To_Staging_Full_Load_CDP_Consumption_MD</t>
         </is>
       </c>
       <c r="B71" t="inlineStr"/>
       <c r="C71" t="inlineStr">
         <is>
-          <t>tFixedFlowInput</t>
+          <t>tImpalaClose</t>
         </is>
       </c>
       <c r="D71" t="inlineStr"/>
@@ -1964,13 +2053,13 @@
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>J_EyeMed_CMS_837_DBLoad_ODS</t>
+          <t>SC_Landing_To_Staging_Full_Load_CDP_Consumption_MD</t>
         </is>
       </c>
       <c r="B72" t="inlineStr"/>
       <c r="C72" t="inlineStr">
         <is>
-          <t>tHashOutput</t>
+          <t>tMysqlClose</t>
         </is>
       </c>
       <c r="D72" t="inlineStr"/>
@@ -1978,13 +2067,13 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>J_EyeMed_CMS_837_DBLoad_ODS</t>
+          <t>SC_Landing_To_Staging_Full_Load_CDP_Consumption_MD</t>
         </is>
       </c>
       <c r="B73" t="inlineStr"/>
       <c r="C73" t="inlineStr">
         <is>
-          <t>tFileCopy</t>
+          <t>Job_Error</t>
         </is>
       </c>
       <c r="D73" t="inlineStr"/>
@@ -1992,13 +2081,13 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>J_EyeMed_CMS_837_DBLoad_ODS</t>
+          <t>SC_Landing_To_Staging_Full_Load_CDP_Consumption_MD</t>
         </is>
       </c>
       <c r="B74" t="inlineStr"/>
       <c r="C74" t="inlineStr">
         <is>
-          <t>tJava</t>
+          <t>tFixedFlowInput</t>
         </is>
       </c>
       <c r="D74" t="inlineStr"/>
@@ -2006,13 +2095,13 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>J_EyeMed_CMS_837_DBLoad_ODS</t>
+          <t>SC_Landing_To_Staging_Full_Load_CDP_Consumption_MD</t>
         </is>
       </c>
       <c r="B75" t="inlineStr"/>
       <c r="C75" t="inlineStr">
         <is>
-          <t>tFileList</t>
+          <t>tFlowToIterate</t>
         </is>
       </c>
       <c r="D75" t="inlineStr"/>
@@ -2020,13 +2109,13 @@
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>J_EyeMed_CMS_837_DBLoad_ODS</t>
+          <t>SC_Landing_To_Staging_Full_Load_CDP_Consumption_MD</t>
         </is>
       </c>
       <c r="B76" t="inlineStr"/>
       <c r="C76" t="inlineStr">
         <is>
-          <t>tFileCopy</t>
+          <t>tImpalaInput</t>
         </is>
       </c>
       <c r="D76" t="inlineStr"/>
@@ -2034,13 +2123,13 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>J_EyeMed_CMS_837_DBLoad_ODS</t>
+          <t>SC_Landing_To_Staging_Full_Load_CDP_Consumption_MD</t>
         </is>
       </c>
       <c r="B77" t="inlineStr"/>
       <c r="C77" t="inlineStr">
         <is>
-          <t>tJava</t>
+          <t>tJavaRow</t>
         </is>
       </c>
       <c r="D77" t="inlineStr"/>
@@ -2048,13 +2137,13 @@
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>J_EyeMed_CMS_837_DBLoad_ODS</t>
+          <t>SC_Landing_To_Staging_Full_Load_CDP_Consumption_MD</t>
         </is>
       </c>
       <c r="B78" t="inlineStr"/>
       <c r="C78" t="inlineStr">
         <is>
-          <t>tMSSqlConnection</t>
+          <t>tImpalaRow</t>
         </is>
       </c>
       <c r="D78" t="inlineStr"/>
@@ -2062,13 +2151,13 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>J_EyeMed_CMS_837_DBLoad_ODS</t>
+          <t>SC_Landing_To_Staging_Full_Load_CDP_Consumption_MD</t>
         </is>
       </c>
       <c r="B79" t="inlineStr"/>
       <c r="C79" t="inlineStr">
         <is>
-          <t>tFileList</t>
+          <t>tImpalaRow</t>
         </is>
       </c>
       <c r="D79" t="inlineStr"/>
@@ -2076,13 +2165,13 @@
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>J_EyeMed_CMS_837_DBLoad_ODS</t>
+          <t>SC_Landing_To_Staging_Full_Load_CDP_Consumption_MD</t>
         </is>
       </c>
       <c r="B80" t="inlineStr"/>
       <c r="C80" t="inlineStr">
         <is>
-          <t>tFileInputRaw</t>
+          <t>tMysqlInput</t>
         </is>
       </c>
       <c r="D80" t="inlineStr"/>
@@ -2090,13 +2179,13 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>J_EyeMed_CMS_837_DBLoad_ODS</t>
+          <t>SC_Landing_To_Staging_Full_Load_CDP_Consumption_MD</t>
         </is>
       </c>
       <c r="B81" t="inlineStr"/>
       <c r="C81" t="inlineStr">
         <is>
-          <t>tHMap</t>
+          <t>tMysqlInput</t>
         </is>
       </c>
       <c r="D81" t="inlineStr"/>
@@ -2104,13 +2193,13 @@
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>J_EyeMed_CMS_837_DBLoad_ODS</t>
+          <t>SC_Landing_To_Staging_Full_Load_CDP_Consumption_MD</t>
         </is>
       </c>
       <c r="B82" t="inlineStr"/>
       <c r="C82" t="inlineStr">
         <is>
-          <t>tFileOutputRaw</t>
+          <t>tImpalaRow</t>
         </is>
       </c>
       <c r="D82" t="inlineStr"/>
@@ -2118,13 +2207,13 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>J_EyeMed_CMS_837_DBLoad_ODS</t>
+          <t>SC_Landing_To_Staging_Full_Load_CDP_Consumption_MD</t>
         </is>
       </c>
       <c r="B83" t="inlineStr"/>
       <c r="C83" t="inlineStr">
         <is>
-          <t>tDie</t>
+          <t>tImpalaRow</t>
         </is>
       </c>
       <c r="D83" t="inlineStr"/>
@@ -2132,13 +2221,13 @@
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>J_EyeMed_CMS_837_DBLoad_ODS</t>
+          <t>SC_Landing_To_Staging_Full_Load_CDP_Consumption_MD</t>
         </is>
       </c>
       <c r="B84" t="inlineStr"/>
       <c r="C84" t="inlineStr">
         <is>
-          <t>tFileList</t>
+          <t>tPrejob</t>
         </is>
       </c>
       <c r="D84" t="inlineStr"/>
@@ -2146,7 +2235,7 @@
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>J_EyeMed_CMS_837_DBLoad_ODS</t>
+          <t>SC_Landing_To_Staging_Full_Load_CDP_Consumption_MD</t>
         </is>
       </c>
       <c r="B85" t="inlineStr"/>
@@ -2160,13 +2249,13 @@
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>J_EyeMed_CMS_837_DBLoad_ODS</t>
+          <t>SC_Landing_To_Staging_Full_Load_CDP_Consumption_MD</t>
         </is>
       </c>
       <c r="B86" t="inlineStr"/>
       <c r="C86" t="inlineStr">
         <is>
-          <t>tMSSqlInput</t>
+          <t>tMysqlConnection</t>
         </is>
       </c>
       <c r="D86" t="inlineStr"/>
@@ -2174,13 +2263,13 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>J_EyeMed_CMS_837_DBLoad_ODS</t>
+          <t>SC_Landing_To_Staging_Full_Load_CDP_Consumption_MD</t>
         </is>
       </c>
       <c r="B87" t="inlineStr"/>
       <c r="C87" t="inlineStr">
         <is>
-          <t>tMap</t>
+          <t>tJava</t>
         </is>
       </c>
       <c r="D87" t="inlineStr"/>
@@ -2188,13 +2277,13 @@
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>J_EyeMed_CMS_837_DBLoad_ODS</t>
+          <t>SC_Landing_To_Staging_Full_Load_CDP_Consumption_MD</t>
         </is>
       </c>
       <c r="B88" t="inlineStr"/>
       <c r="C88" t="inlineStr">
         <is>
-          <t>tSetGlobalVar</t>
+          <t>tMysqlInput</t>
         </is>
       </c>
       <c r="D88" t="inlineStr"/>
@@ -2202,13 +2291,13 @@
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>J_EyeMed_CMS_837_DBLoad_ODS</t>
+          <t>SC_Landing_To_Staging_Full_Load_CDP_Consumption_MD</t>
         </is>
       </c>
       <c r="B89" t="inlineStr"/>
       <c r="C89" t="inlineStr">
         <is>
-          <t>tFileInputXML</t>
+          <t>tFlowToIterate</t>
         </is>
       </c>
       <c r="D89" t="inlineStr"/>
@@ -2216,13 +2305,13 @@
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>J_EyeMed_CMS_837_DBLoad_ODS</t>
+          <t>SC_Landing_To_Staging_Full_Load_CDP_Consumption_MD</t>
         </is>
       </c>
       <c r="B90" t="inlineStr"/>
       <c r="C90" t="inlineStr">
         <is>
-          <t>tMap</t>
+          <t>tJava</t>
         </is>
       </c>
       <c r="D90" t="inlineStr"/>
@@ -2230,13 +2319,13 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>J_EyeMed_CMS_837_DBLoad_ODS</t>
+          <t>SC_Landing_To_Staging_Full_Load_CDP_Consumption_MD</t>
         </is>
       </c>
       <c r="B91" t="inlineStr"/>
       <c r="C91" t="inlineStr">
         <is>
-          <t>tMap</t>
+          <t>tImpalaConnection</t>
         </is>
       </c>
       <c r="D91" t="inlineStr"/>
@@ -2244,13 +2333,13 @@
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>J_EyeMed_CMS_837_DBLoad_ODS</t>
+          <t>SC_Landing_To_Staging_Full_Load_CDP_Consumption_MD</t>
         </is>
       </c>
       <c r="B92" t="inlineStr"/>
       <c r="C92" t="inlineStr">
         <is>
-          <t>tHashInput</t>
+          <t>tImpalaRow</t>
         </is>
       </c>
       <c r="D92" t="inlineStr"/>
@@ -2258,13 +2347,13 @@
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>J_EyeMed_CMS_837_DBLoad_ODS</t>
+          <t>SC_Landing_To_Staging_Full_Load_CDP_Consumption_MD</t>
         </is>
       </c>
       <c r="B93" t="inlineStr"/>
       <c r="C93" t="inlineStr">
         <is>
-          <t>tMSSqlOutput</t>
+          <t>tImpalaInput</t>
         </is>
       </c>
       <c r="D93" t="inlineStr"/>
@@ -2272,13 +2361,13 @@
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>J_EyeMed_CMS_837_DBLoad_ODS</t>
+          <t>SC_Landing_To_Staging_Full_Load_CDP_Consumption_MD</t>
         </is>
       </c>
       <c r="B94" t="inlineStr"/>
       <c r="C94" t="inlineStr">
         <is>
-          <t>tFileInputXML</t>
+          <t>tJavaRow</t>
         </is>
       </c>
       <c r="D94" t="inlineStr"/>
@@ -2286,13 +2375,13 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>J_EyeMed_CMS_837_DBLoad_ODS</t>
+          <t>SC_Landing_To_Staging_Full_Load_CDP_Consumption_MD</t>
         </is>
       </c>
       <c r="B95" t="inlineStr"/>
       <c r="C95" t="inlineStr">
         <is>
-          <t>tMap</t>
+          <t>Job_Start</t>
         </is>
       </c>
       <c r="D95" t="inlineStr"/>
@@ -2300,13 +2389,13 @@
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>J_EyeMed_CMS_837_DBLoad_ODS</t>
+          <t>SC_Landing_To_Staging_Full_Load_CDP_Consumption_MD</t>
         </is>
       </c>
       <c r="B96" t="inlineStr"/>
       <c r="C96" t="inlineStr">
         <is>
-          <t>tMap</t>
+          <t>Implicit_context_joblet</t>
         </is>
       </c>
       <c r="D96" t="inlineStr"/>
@@ -2314,13 +2403,13 @@
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>J_EyeMed_CMS_837_DBLoad_ODS</t>
+          <t>SC_Landing_To_Staging_Full_Load_CDP_Consumption_MD</t>
         </is>
       </c>
       <c r="B97" t="inlineStr"/>
       <c r="C97" t="inlineStr">
         <is>
-          <t>tHashInput</t>
+          <t>tDie</t>
         </is>
       </c>
       <c r="D97" t="inlineStr"/>
@@ -2328,13 +2417,13 @@
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>J_EyeMed_CMS_837_DBLoad_ODS</t>
+          <t>SC_Landing_To_Staging_Full_Load_CDP_Consumption_MD</t>
         </is>
       </c>
       <c r="B98" t="inlineStr"/>
       <c r="C98" t="inlineStr">
         <is>
-          <t>tMSSqlOutput</t>
+          <t>tDie</t>
         </is>
       </c>
       <c r="D98" t="inlineStr"/>
@@ -2342,13 +2431,13 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>J_EyeMed_CMS_837_DBLoad_ODS</t>
+          <t>SC_Landing_To_Staging_Full_Load_CDP_Consumption_MD</t>
         </is>
       </c>
       <c r="B99" t="inlineStr"/>
       <c r="C99" t="inlineStr">
         <is>
-          <t>tFileInputXML</t>
+          <t>tMysqlInput</t>
         </is>
       </c>
       <c r="D99" t="inlineStr"/>
@@ -2356,13 +2445,13 @@
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>J_EyeMed_CMS_837_DBLoad_ODS</t>
+          <t>SC_Landing_To_Staging_Full_Load_CDP_Consumption_MD</t>
         </is>
       </c>
       <c r="B100" t="inlineStr"/>
       <c r="C100" t="inlineStr">
         <is>
-          <t>tMap</t>
+          <t>tJavaRow</t>
         </is>
       </c>
       <c r="D100" t="inlineStr"/>
@@ -2370,13 +2459,13 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>J_EyeMed_CMS_837_DBLoad_ODS</t>
+          <t>SC_Landing_To_Staging_Full_Load_CDP_Consumption_MD</t>
         </is>
       </c>
       <c r="B101" t="inlineStr"/>
       <c r="C101" t="inlineStr">
         <is>
-          <t>tMap</t>
+          <t>tFixedFlowInput</t>
         </is>
       </c>
       <c r="D101" t="inlineStr"/>
@@ -2384,13 +2473,13 @@
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>J_EyeMed_CMS_837_DBLoad_ODS</t>
+          <t>SC_Landing_To_Staging_Full_Load_CDP_Consumption_MD</t>
         </is>
       </c>
       <c r="B102" t="inlineStr"/>
       <c r="C102" t="inlineStr">
         <is>
-          <t>tHashInput</t>
+          <t>tLogRow</t>
         </is>
       </c>
       <c r="D102" t="inlineStr"/>
@@ -2398,13 +2487,13 @@
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>J_EyeMed_CMS_837_DBLoad_ODS</t>
+          <t>SC_Landing_To_Staging_Full_Load_CDP_Consumption_MD</t>
         </is>
       </c>
       <c r="B103" t="inlineStr"/>
       <c r="C103" t="inlineStr">
         <is>
-          <t>tMSSqlOutput</t>
+          <t>tMysqlOutput</t>
         </is>
       </c>
       <c r="D103" t="inlineStr"/>
@@ -2412,13 +2501,13 @@
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>J_EyeMed_CMS_837_DBLoad_ODS</t>
+          <t>SC_Landing_To_Staging_Full_Load_CDP_Consumption_MD</t>
         </is>
       </c>
       <c r="B104" t="inlineStr"/>
       <c r="C104" t="inlineStr">
         <is>
-          <t>tFixedFlowInput</t>
+          <t>Job_End</t>
         </is>
       </c>
       <c r="D104" t="inlineStr"/>
@@ -2426,13 +2515,13 @@
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>J_EyeMed_CMS_837_DBLoad_ODS</t>
+          <t>SC_Landing_To_Staging_Full_Load_CDP_Consumption_MD</t>
         </is>
       </c>
       <c r="B105" t="inlineStr"/>
       <c r="C105" t="inlineStr">
         <is>
-          <t>tJavaRow</t>
+          <t>tMysqlInput</t>
         </is>
       </c>
       <c r="D105" t="inlineStr"/>
@@ -2440,13 +2529,13 @@
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>J_EyeMed_CMS_837_DBLoad_ODS</t>
+          <t>SC_Landing_To_Staging_Full_Load_CDP_Consumption_MD</t>
         </is>
       </c>
       <c r="B106" t="inlineStr"/>
       <c r="C106" t="inlineStr">
         <is>
-          <t>tFileList</t>
+          <t>tFlowToIterate</t>
         </is>
       </c>
       <c r="D106" t="inlineStr"/>
@@ -2454,13 +2543,13 @@
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>J_EyeMed_CMS_837_DBLoad_ODS</t>
+          <t>SC_Landing_To_Staging_Full_Load_CDP_Consumption_MD</t>
         </is>
       </c>
       <c r="B107" t="inlineStr"/>
       <c r="C107" t="inlineStr">
         <is>
-          <t>tFileCopy</t>
+          <t>tMysqlInput</t>
         </is>
       </c>
       <c r="D107" t="inlineStr"/>
@@ -2468,13 +2557,13 @@
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>J_EyeMed_CMS_837_DBLoad_ODS</t>
+          <t>SC_Landing_To_Staging_Full_Load_CDP_Consumption_MD</t>
         </is>
       </c>
       <c r="B108" t="inlineStr"/>
       <c r="C108" t="inlineStr">
         <is>
-          <t>tJava</t>
+          <t>tJavaRow</t>
         </is>
       </c>
       <c r="D108" t="inlineStr"/>
@@ -2482,7 +2571,7 @@
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>J_EyeMed_CMS_837_DBLoad_ODS</t>
+          <t>SC_Landing_To_Staging_Full_Load_CDP_Consumption_MD</t>
         </is>
       </c>
       <c r="B109" t="inlineStr"/>
@@ -2496,13 +2585,13 @@
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>J_EyeMed_CMS_837_DBLoad_ODS</t>
+          <t>SC_Landing_To_Staging_Full_Load_CDP_Consumption_MD</t>
         </is>
       </c>
       <c r="B110" t="inlineStr"/>
       <c r="C110" t="inlineStr">
         <is>
-          <t>tFileInputXML</t>
+          <t>tImpalaRow</t>
         </is>
       </c>
       <c r="D110" t="inlineStr"/>
@@ -2510,13 +2599,13 @@
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>J_EyeMed_CMS_837_DBLoad_ODS</t>
+          <t>SC_Landing_To_Staging_Full_Load_CDP_Consumption_MD</t>
         </is>
       </c>
       <c r="B111" t="inlineStr"/>
       <c r="C111" t="inlineStr">
         <is>
-          <t>tMap</t>
+          <t>tPostjob</t>
         </is>
       </c>
       <c r="D111" t="inlineStr"/>
@@ -2524,13 +2613,13 @@
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>J_EyeMed_CMS_837_DBLoad_ODS</t>
+          <t>SC_Landing_To_Staging_Full_Load_CDP_Consumption_MD</t>
         </is>
       </c>
       <c r="B112" t="inlineStr"/>
       <c r="C112" t="inlineStr">
         <is>
-          <t>tMap</t>
+          <t>tImpalaClose</t>
         </is>
       </c>
       <c r="D112" t="inlineStr"/>
@@ -2538,13 +2627,13 @@
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>J_EyeMed_CMS_837_DBLoad_ODS</t>
+          <t>SC_Landing_To_Staging_Full_Load_CDP_Consumption_MD</t>
         </is>
       </c>
       <c r="B113" t="inlineStr"/>
       <c r="C113" t="inlineStr">
         <is>
-          <t>tMSSqlOutput</t>
+          <t>tMysqlClose</t>
         </is>
       </c>
       <c r="D113" t="inlineStr"/>
@@ -2552,13 +2641,13 @@
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>J_EyeMed_CMS_837_DBLoad_ODS</t>
+          <t>SC_Landing_To_Staging_Full_Load_CDP_Consumption_MD</t>
         </is>
       </c>
       <c r="B114" t="inlineStr"/>
       <c r="C114" t="inlineStr">
         <is>
-          <t>tFileInputDelimited</t>
+          <t>Job_Error</t>
         </is>
       </c>
       <c r="D114" t="inlineStr"/>
@@ -2566,13 +2655,13 @@
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>J_EyeMed_CMS_837_DBLoad_ODS</t>
+          <t>SC_Landing_To_Staging_Full_Load_CDP_Consumption_MD</t>
         </is>
       </c>
       <c r="B115" t="inlineStr"/>
       <c r="C115" t="inlineStr">
         <is>
-          <t>tJavaRow</t>
+          <t>tFixedFlowInput</t>
         </is>
       </c>
       <c r="D115" t="inlineStr"/>
@@ -2580,13 +2669,13 @@
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>J_EyeMed_CMS_837_DBLoad_ODS</t>
+          <t>SC_Landing_To_Staging_Full_Load_CDP_Consumption_MD</t>
         </is>
       </c>
       <c r="B116" t="inlineStr"/>
       <c r="C116" t="inlineStr">
         <is>
-          <t>tFileInputXML</t>
+          <t>tFlowToIterate</t>
         </is>
       </c>
       <c r="D116" t="inlineStr"/>
@@ -2594,13 +2683,13 @@
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t>J_EyeMed_CMS_837_DBLoad_ODS</t>
+          <t>SC_Landing_To_Staging_Full_Load_CDP_Consumption_MD</t>
         </is>
       </c>
       <c r="B117" t="inlineStr"/>
       <c r="C117" t="inlineStr">
         <is>
-          <t>tMap</t>
+          <t>tImpalaInput</t>
         </is>
       </c>
       <c r="D117" t="inlineStr"/>
@@ -2608,13 +2697,13 @@
     <row r="118">
       <c r="A118" t="inlineStr">
         <is>
-          <t>J_EyeMed_CMS_837_DBLoad_ODS</t>
+          <t>SC_Landing_To_Staging_Full_Load_CDP_Consumption_MD</t>
         </is>
       </c>
       <c r="B118" t="inlineStr"/>
       <c r="C118" t="inlineStr">
         <is>
-          <t>tMap</t>
+          <t>tJavaRow</t>
         </is>
       </c>
       <c r="D118" t="inlineStr"/>
@@ -2622,13 +2711,13 @@
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
-          <t>J_EyeMed_CMS_837_DBLoad_ODS</t>
+          <t>SC_Landing_To_Staging_Full_Load_CDP_Consumption_MD</t>
         </is>
       </c>
       <c r="B119" t="inlineStr"/>
       <c r="C119" t="inlineStr">
         <is>
-          <t>tMSSqlInput</t>
+          <t>tImpalaRow</t>
         </is>
       </c>
       <c r="D119" t="inlineStr"/>
@@ -2636,13 +2725,13 @@
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>J_EyeMed_CMS_837_DBLoad_ODS</t>
+          <t>SC_Landing_To_Staging_Full_Load_CDP_Consumption_MD</t>
         </is>
       </c>
       <c r="B120" t="inlineStr"/>
       <c r="C120" t="inlineStr">
         <is>
-          <t>tMSSqlOutput</t>
+          <t>tImpalaRow</t>
         </is>
       </c>
       <c r="D120" t="inlineStr"/>
@@ -2650,13 +2739,13 @@
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>J_EyeMed_CMS_837_DBLoad_ODS</t>
+          <t>SC_Landing_To_Staging_Full_Load_CDP_Consumption_MD</t>
         </is>
       </c>
       <c r="B121" t="inlineStr"/>
       <c r="C121" t="inlineStr">
         <is>
-          <t>tFTPConnection</t>
+          <t>tMysqlInput</t>
         </is>
       </c>
       <c r="D121" t="inlineStr"/>
@@ -2664,13 +2753,13 @@
     <row r="122">
       <c r="A122" t="inlineStr">
         <is>
-          <t>J_EyeMed_CMS_837_DBLoad_ODS</t>
+          <t>SC_Landing_To_Staging_Full_Load_CDP_Consumption_MD</t>
         </is>
       </c>
       <c r="B122" t="inlineStr"/>
       <c r="C122" t="inlineStr">
         <is>
-          <t>tFTPFileList</t>
+          <t>tMysqlInput</t>
         </is>
       </c>
       <c r="D122" t="inlineStr"/>
@@ -2678,13 +2767,13 @@
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
-          <t>J_EyeMed_CMS_837_DBLoad_ODS</t>
+          <t>SC_Landing_To_Staging_Full_Load_CDP_Consumption_MD</t>
         </is>
       </c>
       <c r="B123" t="inlineStr"/>
       <c r="C123" t="inlineStr">
         <is>
-          <t>tFTPGet</t>
+          <t>tImpalaRow</t>
         </is>
       </c>
       <c r="D123" t="inlineStr"/>
@@ -2692,13 +2781,13 @@
     <row r="124">
       <c r="A124" t="inlineStr">
         <is>
-          <t>J_EyeMed_CMS_837_DBLoad_ODS</t>
+          <t>SC_Landing_To_Staging_Full_Load_CDP_Consumption_MD</t>
         </is>
       </c>
       <c r="B124" t="inlineStr"/>
       <c r="C124" t="inlineStr">
         <is>
-          <t>tSendMail</t>
+          <t>tImpalaRow</t>
         </is>
       </c>
       <c r="D124" t="inlineStr"/>
@@ -2706,13 +2795,13 @@
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>J_EyeMed_CMS_837_DBLoad_ODS</t>
+          <t>SC_Landing_To_Staging_Full_Load_CDP_Consumption_MD</t>
         </is>
       </c>
       <c r="B125" t="inlineStr"/>
       <c r="C125" t="inlineStr">
         <is>
-          <t>tSendMail</t>
+          <t>tImpalaRow</t>
         </is>
       </c>
       <c r="D125" t="inlineStr"/>
@@ -2720,13 +2809,13 @@
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>J_EyeMed_CMS_837_DBLoad_ODS</t>
+          <t>SC_Landing_To_Staging_Full_Load_CDP_Consumption_MD</t>
         </is>
       </c>
       <c r="B126" t="inlineStr"/>
       <c r="C126" t="inlineStr">
         <is>
-          <t>tDie</t>
+          <t>tImpalaRow</t>
         </is>
       </c>
       <c r="D126" t="inlineStr"/>
@@ -2734,13 +2823,13 @@
     <row r="127">
       <c r="A127" t="inlineStr">
         <is>
-          <t>J_EyeMed_CMS_837_DBLoad_ODS</t>
+          <t>SC_Landing_To_Staging_Full_Load_CDP_Consumption_MD</t>
         </is>
       </c>
       <c r="B127" t="inlineStr"/>
       <c r="C127" t="inlineStr">
         <is>
-          <t>tPrejob</t>
+          <t>tFixedFlowInput</t>
         </is>
       </c>
       <c r="D127" t="inlineStr"/>
@@ -2748,13 +2837,13 @@
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
-          <t>J_EyeMed_CMS_837_DBLoad_ODS</t>
+          <t>SC_Landing_To_Staging_Full_Load_CDP_Consumption_MD</t>
         </is>
       </c>
       <c r="B128" t="inlineStr"/>
       <c r="C128" t="inlineStr">
         <is>
-          <t>tMSSqlConnection</t>
+          <t>tFlowToIterate</t>
         </is>
       </c>
       <c r="D128" t="inlineStr"/>
@@ -2762,13 +2851,13 @@
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t>J_EyeMed_CMS_837_DBLoad_ODS</t>
+          <t>SC_Landing_To_Staging_Full_Load_CDP_Consumption_MD</t>
         </is>
       </c>
       <c r="B129" t="inlineStr"/>
       <c r="C129" t="inlineStr">
         <is>
-          <t>tStatCatcher</t>
+          <t>tImpalaInput</t>
         </is>
       </c>
       <c r="D129" t="inlineStr"/>
@@ -2776,13 +2865,13 @@
     <row r="130">
       <c r="A130" t="inlineStr">
         <is>
-          <t>J_EyeMed_CMS_837_DBLoad_ODS</t>
+          <t>SC_Landing_To_Staging_Full_Load_CDP_Consumption_MD</t>
         </is>
       </c>
       <c r="B130" t="inlineStr"/>
       <c r="C130" t="inlineStr">
         <is>
-          <t>tMap</t>
+          <t>tJavaRow</t>
         </is>
       </c>
       <c r="D130" t="inlineStr"/>
@@ -2790,13 +2879,13 @@
     <row r="131">
       <c r="A131" t="inlineStr">
         <is>
-          <t>J_EyeMed_CMS_837_DBLoad_ODS</t>
+          <t>SC_Landing_To_Staging_Full_Load_CDP_Consumption_MD</t>
         </is>
       </c>
       <c r="B131" t="inlineStr"/>
       <c r="C131" t="inlineStr">
         <is>
-          <t>tFlowToIterate</t>
+          <t>tHiveConnection</t>
         </is>
       </c>
       <c r="D131" t="inlineStr"/>
@@ -2804,13 +2893,13 @@
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>J_EyeMed_CMS_837_DBLoad_ODS</t>
+          <t>SC_Landing_To_Staging_Full_Load_CDP_Consumption_MD</t>
         </is>
       </c>
       <c r="B132" t="inlineStr"/>
       <c r="C132" t="inlineStr">
         <is>
-          <t>tJavaRow</t>
+          <t>tHiveRow</t>
         </is>
       </c>
       <c r="D132" t="inlineStr"/>
@@ -2818,13 +2907,13 @@
     <row r="133">
       <c r="A133" t="inlineStr">
         <is>
-          <t>J_EyeMed_CMS_837_DBLoad_ODS</t>
+          <t>SC_Landing_To_Staging_Full_Load_CDP_Consumption_MD</t>
         </is>
       </c>
       <c r="B133" t="inlineStr"/>
       <c r="C133" t="inlineStr">
         <is>
-          <t>tMSSqlOutput</t>
+          <t>tHiveRow</t>
         </is>
       </c>
       <c r="D133" t="inlineStr"/>
@@ -2832,13 +2921,13 @@
     <row r="134">
       <c r="A134" t="inlineStr">
         <is>
-          <t>J_EyeMed_CMS_837_DBLoad_ODS</t>
+          <t>SC_Landing_To_Staging_Full_Load_CDP_Consumption_MD</t>
         </is>
       </c>
       <c r="B134" t="inlineStr"/>
       <c r="C134" t="inlineStr">
         <is>
-          <t>tSendMail</t>
+          <t>tHiveConnection</t>
         </is>
       </c>
       <c r="D134" t="inlineStr"/>
@@ -2846,13 +2935,13 @@
     <row r="135">
       <c r="A135" t="inlineStr">
         <is>
-          <t>J_EyeMed_CMS_837_DBLoad_ODS</t>
+          <t>SC_Landing_To_Staging_Full_Load_CDP_Consumption_MD</t>
         </is>
       </c>
       <c r="B135" t="inlineStr"/>
       <c r="C135" t="inlineStr">
         <is>
-          <t>tLogCatcher</t>
+          <t>tHiveInput</t>
         </is>
       </c>
       <c r="D135" t="inlineStr"/>
@@ -2860,13 +2949,13 @@
     <row r="136">
       <c r="A136" t="inlineStr">
         <is>
-          <t>J_EyeMed_CMS_837_DBLoad_ODS</t>
+          <t>SC_Landing_To_Staging_Full_Load_CDP_Consumption_MD</t>
         </is>
       </c>
       <c r="B136" t="inlineStr"/>
       <c r="C136" t="inlineStr">
         <is>
-          <t>tMap</t>
+          <t>tJavaRow</t>
         </is>
       </c>
       <c r="D136" t="inlineStr"/>
@@ -2874,13 +2963,13 @@
     <row r="137">
       <c r="A137" t="inlineStr">
         <is>
-          <t>J_EyeMed_CMS_837_DBLoad_ODS</t>
+          <t>SC_Landing_To_Staging_Full_Load_CDP_Consumption_MD</t>
         </is>
       </c>
       <c r="B137" t="inlineStr"/>
       <c r="C137" t="inlineStr">
         <is>
-          <t>tFlowToIterate</t>
+          <t>tHiveConnection</t>
         </is>
       </c>
       <c r="D137" t="inlineStr"/>
@@ -2888,13 +2977,13 @@
     <row r="138">
       <c r="A138" t="inlineStr">
         <is>
-          <t>J_EyeMed_CMS_837_DBLoad_ODS</t>
+          <t>SC_Landing_To_Staging_Full_Load_CDP_Consumption_MD</t>
         </is>
       </c>
       <c r="B138" t="inlineStr"/>
       <c r="C138" t="inlineStr">
         <is>
-          <t>tMSSqlOutput</t>
+          <t>tHiveConnection</t>
         </is>
       </c>
       <c r="D138" t="inlineStr"/>
@@ -2902,13 +2991,13 @@
     <row r="139">
       <c r="A139" t="inlineStr">
         <is>
-          <t>J_EyeMed_CMS_837_DBLoad_ODS</t>
+          <t>SC_Landing_To_Staging_Full_Load_CDP_Consumption_MD</t>
         </is>
       </c>
       <c r="B139" t="inlineStr"/>
       <c r="C139" t="inlineStr">
         <is>
-          <t>tSendMail</t>
+          <t>tHiveInput</t>
         </is>
       </c>
       <c r="D139" t="inlineStr"/>
@@ -2916,13 +3005,13 @@
     <row r="140">
       <c r="A140" t="inlineStr">
         <is>
-          <t>J_EyeMed_CMS_837_DBLoad_ODS</t>
+          <t>SC_Landing_To_Staging_Full_Load_CDP_Consumption_MD</t>
         </is>
       </c>
       <c r="B140" t="inlineStr"/>
       <c r="C140" t="inlineStr">
         <is>
-          <t>tDie</t>
+          <t>tJavaRow</t>
         </is>
       </c>
       <c r="D140" t="inlineStr"/>
@@ -2930,13 +3019,13 @@
     <row r="141">
       <c r="A141" t="inlineStr">
         <is>
-          <t>J_EyeMed_CMS_837_DBLoad_ODS</t>
+          <t>SC_Landing_To_Staging_Full_Load_CDP_Consumption_MD</t>
         </is>
       </c>
       <c r="B141" t="inlineStr"/>
       <c r="C141" t="inlineStr">
         <is>
-          <t>tFTPDelete</t>
+          <t>tJava</t>
         </is>
       </c>
       <c r="D141" t="inlineStr"/>
@@ -2944,13 +3033,13 @@
     <row r="142">
       <c r="A142" t="inlineStr">
         <is>
-          <t>J_EyeMed_CMS_837_DBLoad_ODS</t>
+          <t>SC_Landing_To_Staging_Full_Load_CDP_Consumption_MD</t>
         </is>
       </c>
       <c r="B142" t="inlineStr"/>
       <c r="C142" t="inlineStr">
         <is>
-          <t>tFileInputXML</t>
+          <t>tJava</t>
         </is>
       </c>
       <c r="D142" t="inlineStr"/>
@@ -2958,13 +3047,13 @@
     <row r="143">
       <c r="A143" t="inlineStr">
         <is>
-          <t>J_EyeMed_CMS_837_DBLoad_ODS</t>
+          <t>SC_Landing_To_Staging_Full_Load_CDP_Consumption_MD</t>
         </is>
       </c>
       <c r="B143" t="inlineStr"/>
       <c r="C143" t="inlineStr">
         <is>
-          <t>tMap</t>
+          <t>tImpalaRow</t>
         </is>
       </c>
       <c r="D143" t="inlineStr"/>
@@ -2972,13 +3061,13 @@
     <row r="144">
       <c r="A144" t="inlineStr">
         <is>
-          <t>J_EyeMed_CMS_837_DBLoad_ODS</t>
+          <t>SC_Landing_To_Staging_Full_Load_CDP_Consumption_MD</t>
         </is>
       </c>
       <c r="B144" t="inlineStr"/>
       <c r="C144" t="inlineStr">
         <is>
-          <t>tHashOutput</t>
+          <t>tImpalaRow</t>
         </is>
       </c>
       <c r="D144" t="inlineStr"/>
@@ -2986,13 +3075,13 @@
     <row r="145">
       <c r="A145" t="inlineStr">
         <is>
-          <t>J_EyeMed_CMS_837_DBLoad_ODS</t>
+          <t>SC_Landing_To_Staging_Full_Load_CDP_Consumption_MD</t>
         </is>
       </c>
       <c r="B145" t="inlineStr"/>
       <c r="C145" t="inlineStr">
         <is>
-          <t>tPostjob</t>
+          <t>tImpalaRow</t>
         </is>
       </c>
       <c r="D145" t="inlineStr"/>
@@ -3000,13 +3089,13 @@
     <row r="146">
       <c r="A146" t="inlineStr">
         <is>
-          <t>J_EyeMed_CMS_837_DBLoad_ODS</t>
+          <t>SC_Landing_To_Staging_Full_Load_CDP_Consumption_MD</t>
         </is>
       </c>
       <c r="B146" t="inlineStr"/>
       <c r="C146" t="inlineStr">
         <is>
-          <t>tMSSqlClose</t>
+          <t>tImpalaRow</t>
         </is>
       </c>
       <c r="D146" t="inlineStr"/>
@@ -3014,13 +3103,13 @@
     <row r="147">
       <c r="A147" t="inlineStr">
         <is>
-          <t>J_EyeMed_CMS_837_DBLoad_ODS</t>
+          <t>SC_Landing_To_Staging_Full_Load_CDP_Consumption_MD</t>
         </is>
       </c>
       <c r="B147" t="inlineStr"/>
       <c r="C147" t="inlineStr">
         <is>
-          <t>tFixedFlowInput</t>
+          <t>tImpalaConnection</t>
         </is>
       </c>
       <c r="D147" t="inlineStr"/>
@@ -3028,13 +3117,13 @@
     <row r="148">
       <c r="A148" t="inlineStr">
         <is>
-          <t>J_EyeMed_CMS_837_DBLoad_ODS</t>
+          <t>SC_Landing_To_Staging_Full_Load_CDP_Consumption_MD</t>
         </is>
       </c>
       <c r="B148" t="inlineStr"/>
       <c r="C148" t="inlineStr">
         <is>
-          <t>tHashOutput</t>
+          <t>tDie</t>
         </is>
       </c>
       <c r="D148" t="inlineStr"/>
@@ -3042,13 +3131,13 @@
     <row r="149">
       <c r="A149" t="inlineStr">
         <is>
-          <t>J_EyeMed_CMS_837_DBLoad_ODS</t>
+          <t>SC_Landing_To_Staging_Full_Load_CDP_Consumption_MD</t>
         </is>
       </c>
       <c r="B149" t="inlineStr"/>
       <c r="C149" t="inlineStr">
         <is>
-          <t>tFileCopy</t>
+          <t>tFixedFlowInput</t>
         </is>
       </c>
       <c r="D149" t="inlineStr"/>
@@ -3056,13 +3145,13 @@
     <row r="150">
       <c r="A150" t="inlineStr">
         <is>
-          <t>J_EyeMed_CMS_837_DBLoad_ODS</t>
+          <t>SC_Landing_To_Staging_Full_Load_CDP_Consumption_MD</t>
         </is>
       </c>
       <c r="B150" t="inlineStr"/>
       <c r="C150" t="inlineStr">
         <is>
-          <t>tJava</t>
+          <t>tFixedFlowInput</t>
         </is>
       </c>
       <c r="D150" t="inlineStr"/>
@@ -3070,13 +3159,13 @@
     <row r="151">
       <c r="A151" t="inlineStr">
         <is>
-          <t>J_EyeMed_CMS_837_DBLoad_ODS</t>
+          <t>SC_Landing_To_Staging_Full_Load_CDP_Consumption_MD</t>
         </is>
       </c>
       <c r="B151" t="inlineStr"/>
       <c r="C151" t="inlineStr">
         <is>
-          <t>tFileList</t>
+          <t>tFlowToIterate</t>
         </is>
       </c>
       <c r="D151" t="inlineStr"/>
@@ -3084,13 +3173,13 @@
     <row r="152">
       <c r="A152" t="inlineStr">
         <is>
-          <t>J_EyeMed_CMS_837_DBLoad_ODS</t>
+          <t>SC_Landing_To_Staging_Full_Load_CDP_Consumption_MD</t>
         </is>
       </c>
       <c r="B152" t="inlineStr"/>
       <c r="C152" t="inlineStr">
         <is>
-          <t>tFileCopy</t>
+          <t>tHiveRow</t>
         </is>
       </c>
       <c r="D152" t="inlineStr"/>
@@ -3098,13 +3187,13 @@
     <row r="153">
       <c r="A153" t="inlineStr">
         <is>
-          <t>J_EyeMed_CMS_837_DBLoad_ODS</t>
+          <t>SC_Landing_To_Staging_Full_Load_CDP_Consumption_MD</t>
         </is>
       </c>
       <c r="B153" t="inlineStr"/>
       <c r="C153" t="inlineStr">
         <is>
-          <t>tJava</t>
+          <t>tHiveRow</t>
         </is>
       </c>
       <c r="D153" t="inlineStr"/>
@@ -3120,10 +3209,10 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D17"/>
+  <dimension ref="A1:D27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="29" customWidth="1" min="1" max="1"/>
+    <col width="52" customWidth="1" min="1" max="1"/>
     <col width="60" customWidth="1" min="2" max="2"/>
     <col width="10" customWidth="1" min="3" max="3"/>
     <col width="10" customWidth="1" min="4" max="4"/>
@@ -3154,7 +3243,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>J_EyeMed_CMS_837_DBLoad_ODS</t>
+          <t>SC_Landing_To_Staging_Full_Load_CDP_Consumption_MD</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -3172,12 +3261,12 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>J_EyeMed_CMS_837_DBLoad_ODS</t>
+          <t>SC_Landing_To_Staging_Full_Load_CDP_Consumption_MD</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>{'component': 'tJavaRow', 'risk': 'HIGH', 'modernization': 'Replace with tMap expressions', 'replacement': 'tMap'}</t>
+          <t>{'component': 'tJava', 'risk': 'HIGH', 'modernization': 'Rewrite using Talend native components', 'replacement': 'tMap / Talend Routine'}</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -3190,7 +3279,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>J_EyeMed_CMS_837_DBLoad_ODS</t>
+          <t>SC_Landing_To_Staging_Full_Load_CDP_Consumption_MD</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -3208,7 +3297,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>J_EyeMed_CMS_837_DBLoad_ODS</t>
+          <t>SC_Landing_To_Staging_Full_Load_CDP_Consumption_MD</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -3226,12 +3315,12 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>J_EyeMed_CMS_837_DBLoad_ODS</t>
+          <t>SC_Landing_To_Staging_Full_Load_CDP_Consumption_MD</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>{'component': 'tFTPGet', 'risk': 'MEDIUM', 'modernization': 'Replace with secure file transfer', 'replacement': 'tFTPFileList'}</t>
+          <t>{'component': 'tJavaRow', 'risk': 'HIGH', 'modernization': 'Replace with tMap expressions', 'replacement': 'tMap'}</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -3244,7 +3333,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>J_EyeMed_CMS_837_DBLoad_ODS</t>
+          <t>SC_Landing_To_Staging_Full_Load_CDP_Consumption_MD</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -3262,12 +3351,12 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>J_EyeMed_CMS_837_DBLoad_ODS</t>
+          <t>SC_Landing_To_Staging_Full_Load_CDP_Consumption_MD</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>{'component': 'tJava', 'risk': 'HIGH', 'modernization': 'Rewrite using Talend native components', 'replacement': 'tMap / Talend Routine'}</t>
+          <t>{'component': 'tJavaRow', 'risk': 'HIGH', 'modernization': 'Replace with tMap expressions', 'replacement': 'tMap'}</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -3280,7 +3369,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>J_EyeMed_CMS_837_DBLoad_ODS</t>
+          <t>SC_Landing_To_Staging_Full_Load_CDP_Consumption_MD</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -3298,7 +3387,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>J_EyeMed_CMS_837_DBLoad_ODS</t>
+          <t>SC_Landing_To_Staging_Full_Load_CDP_Consumption_MD</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -3316,12 +3405,12 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>J_EyeMed_CMS_837_DBLoad_ODS</t>
+          <t>SC_Landing_To_Staging_Full_Load_CDP_Consumption_MD</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>{'component': 'tJavaRow', 'risk': 'HIGH', 'modernization': 'Replace with tMap expressions', 'replacement': 'tMap'}</t>
+          <t>{'component': 'tJava', 'risk': 'HIGH', 'modernization': 'Rewrite using Talend native components', 'replacement': 'tMap / Talend Routine'}</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -3334,12 +3423,12 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>J_EyeMed_CMS_837_DBLoad_ODS</t>
+          <t>SC_Landing_To_Staging_Full_Load_CDP_Consumption_MD</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>{'component': 'tJava', 'risk': 'HIGH', 'modernization': 'Rewrite using Talend native components', 'replacement': 'tMap / Talend Routine'}</t>
+          <t>{'component': 'tJavaRow', 'risk': 'HIGH', 'modernization': 'Replace with tMap expressions', 'replacement': 'tMap'}</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -3352,7 +3441,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>J_EyeMed_CMS_837_DBLoad_ODS</t>
+          <t>SC_Landing_To_Staging_Full_Load_CDP_Consumption_MD</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -3370,12 +3459,12 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>J_EyeMed_CMS_837_DBLoad_ODS</t>
+          <t>SC_Landing_To_Staging_Full_Load_CDP_Consumption_MD</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>{'component': 'tFTPGet', 'risk': 'MEDIUM', 'modernization': 'Replace with secure file transfer', 'replacement': 'tFTPFileList'}</t>
+          <t>{'component': 'tJavaRow', 'risk': 'HIGH', 'modernization': 'Replace with tMap expressions', 'replacement': 'tMap'}</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -3388,7 +3477,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>J_EyeMed_CMS_837_DBLoad_ODS</t>
+          <t>SC_Landing_To_Staging_Full_Load_CDP_Consumption_MD</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -3406,7 +3495,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>J_EyeMed_CMS_837_DBLoad_ODS</t>
+          <t>SC_Landing_To_Staging_Full_Load_CDP_Consumption_MD</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -3424,7 +3513,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>J_EyeMed_CMS_837_DBLoad_ODS</t>
+          <t>SC_Landing_To_Staging_Full_Load_CDP_Consumption_MD</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -3438,6 +3527,186 @@
         </is>
       </c>
       <c r="D17" t="inlineStr"/>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>SC_Landing_To_Staging_Full_Load_CDP_Consumption_MD</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>{'component': 'tJava', 'risk': 'HIGH', 'modernization': 'Rewrite using Talend native components', 'replacement': 'tMap / Talend Routine'}</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>SC_Landing_To_Staging_Full_Load_CDP_Consumption_MD</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>{'component': 'tJavaRow', 'risk': 'HIGH', 'modernization': 'Replace with tMap expressions', 'replacement': 'tMap'}</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr"/>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>SC_Landing_To_Staging_Full_Load_CDP_Consumption_MD</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>{'component': 'tJavaRow', 'risk': 'HIGH', 'modernization': 'Replace with tMap expressions', 'replacement': 'tMap'}</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr"/>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>SC_Landing_To_Staging_Full_Load_CDP_Consumption_MD</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>{'component': 'tJavaRow', 'risk': 'HIGH', 'modernization': 'Replace with tMap expressions', 'replacement': 'tMap'}</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr"/>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>SC_Landing_To_Staging_Full_Load_CDP_Consumption_MD</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>{'component': 'tJavaRow', 'risk': 'HIGH', 'modernization': 'Replace with tMap expressions', 'replacement': 'tMap'}</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr"/>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>SC_Landing_To_Staging_Full_Load_CDP_Consumption_MD</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>{'component': 'tJavaRow', 'risk': 'HIGH', 'modernization': 'Replace with tMap expressions', 'replacement': 'tMap'}</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr"/>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>SC_Landing_To_Staging_Full_Load_CDP_Consumption_MD</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>{'component': 'tJavaRow', 'risk': 'HIGH', 'modernization': 'Replace with tMap expressions', 'replacement': 'tMap'}</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr"/>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>SC_Landing_To_Staging_Full_Load_CDP_Consumption_MD</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>{'component': 'tJavaRow', 'risk': 'HIGH', 'modernization': 'Replace with tMap expressions', 'replacement': 'tMap'}</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr"/>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>SC_Landing_To_Staging_Full_Load_CDP_Consumption_MD</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>{'component': 'tJava', 'risk': 'HIGH', 'modernization': 'Rewrite using Talend native components', 'replacement': 'tMap / Talend Routine'}</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr"/>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>SC_Landing_To_Staging_Full_Load_CDP_Consumption_MD</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>{'component': 'tJava', 'risk': 'HIGH', 'modernization': 'Rewrite using Talend native components', 'replacement': 'tMap / Talend Routine'}</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>